<commit_message>
Inventario de cierre Viñas Norte: resumen con fórmulas de Estado + historial diario por lote
- Resumen Actual: Estado con fórmulas IF (AGOTADO/CRÍTICO/BAJO/OK) y formato condicional
- Historial Lote 34/9/10: salida diaria y saldo restante por material, ponderado por asistencia de piseros

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXSZ5Q2QVHttNZRkf7MNkK
</commit_message>
<xml_diff>
--- a/Viñas Norte - Inventario y Historial (cierre).xlsx
+++ b/Viñas Norte - Inventario y Historial (cierre).xlsx
@@ -50,7 +50,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +75,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3CF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -114,14 +119,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -133,31 +138,83 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="001E8449"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D5F5E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B7950B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCF3CF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00922B21"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F5B7B1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00566573"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D5D8DC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -526,7 +583,7 @@
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -589,10 +646,9 @@
       <c r="D7" s="7" t="n">
         <v>48</v>
       </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+      <c r="E7" s="8">
+        <f>IF(D7=0,"AGOTADO",IF(D7/C7&lt;=0.15,"CRÍTICO",IF(D7/C7&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F7" s="5" t="n"/>
     </row>
@@ -608,10 +664,9 @@
       <c r="D8" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E8" s="8">
+        <f>IF(D8=0,"AGOTADO",IF(D8/C8&lt;=0.15,"CRÍTICO",IF(D8/C8&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F8" s="5" t="n"/>
     </row>
@@ -627,10 +682,9 @@
       <c r="D9" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+      <c r="E9" s="8">
+        <f>IF(D9=0,"AGOTADO",IF(D9/C9&lt;=0.15,"CRÍTICO",IF(D9/C9&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F9" s="5" t="n"/>
     </row>
@@ -646,10 +700,9 @@
       <c r="D10" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+      <c r="E10" s="8">
+        <f>IF(D10=0,"AGOTADO",IF(D10/C10&lt;=0.15,"CRÍTICO",IF(D10/C10&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F10" s="5" t="n"/>
     </row>
@@ -665,10 +718,9 @@
       <c r="D11" s="7" t="n">
         <v>41</v>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+      <c r="E11" s="8">
+        <f>IF(D11=0,"AGOTADO",IF(D11/C11&lt;=0.15,"CRÍTICO",IF(D11/C11&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F11" s="5" t="n"/>
     </row>
@@ -684,10 +736,9 @@
       <c r="D12" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>BAJO</t>
-        </is>
+      <c r="E12" s="8">
+        <f>IF(D12=0,"AGOTADO",IF(D12/C12&lt;=0.15,"CRÍTICO",IF(D12/C12&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F12" s="5" t="n"/>
     </row>
@@ -737,10 +788,9 @@
       <c r="D16" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E16" s="8">
+        <f>IF(D16=0,"AGOTADO",IF(D16/C16&lt;=0.15,"CRÍTICO",IF(D16/C16&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F16" s="5" t="n"/>
     </row>
@@ -756,10 +806,9 @@
       <c r="D17" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E17" s="8">
+        <f>IF(D17=0,"AGOTADO",IF(D17/C17&lt;=0.15,"CRÍTICO",IF(D17/C17&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F17" s="5" t="n"/>
     </row>
@@ -775,10 +824,9 @@
       <c r="D18" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E18" s="8">
+        <f>IF(D18=0,"AGOTADO",IF(D18/C18&lt;=0.15,"CRÍTICO",IF(D18/C18&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F18" s="5" t="n"/>
     </row>
@@ -794,10 +842,9 @@
       <c r="D19" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E19" s="8">
+        <f>IF(D19=0,"AGOTADO",IF(D19/C19&lt;=0.15,"CRÍTICO",IF(D19/C19&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F19" s="5" t="n"/>
     </row>
@@ -813,10 +860,9 @@
       <c r="D20" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E20" s="8">
+        <f>IF(D20=0,"AGOTADO",IF(D20/C20&lt;=0.15,"CRÍTICO",IF(D20/C20&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F20" s="5" t="n"/>
     </row>
@@ -832,10 +878,9 @@
       <c r="D21" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E21" s="8">
+        <f>IF(D21=0,"AGOTADO",IF(D21/C21&lt;=0.15,"CRÍTICO",IF(D21/C21&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F21" s="5" t="n"/>
     </row>
@@ -885,10 +930,9 @@
       <c r="D25" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E25" s="8">
+        <f>IF(D25=0,"AGOTADO",IF(D25/C25&lt;=0.15,"CRÍTICO",IF(D25/C25&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F25" s="5" t="n"/>
     </row>
@@ -904,10 +948,9 @@
       <c r="D26" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E26" s="8">
+        <f>IF(D26=0,"AGOTADO",IF(D26/C26&lt;=0.15,"CRÍTICO",IF(D26/C26&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F26" s="5" t="n"/>
     </row>
@@ -923,10 +966,9 @@
       <c r="D27" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+      <c r="E27" s="8">
+        <f>IF(D27=0,"AGOTADO",IF(D27/C27&lt;=0.15,"CRÍTICO",IF(D27/C27&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F27" s="5" t="n"/>
     </row>
@@ -942,10 +984,9 @@
       <c r="D28" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E28" s="8">
+        <f>IF(D28=0,"AGOTADO",IF(D28/C28&lt;=0.15,"CRÍTICO",IF(D28/C28&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F28" s="5" t="n"/>
     </row>
@@ -961,10 +1002,9 @@
       <c r="D29" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E29" s="8">
+        <f>IF(D29=0,"AGOTADO",IF(D29/C29&lt;=0.15,"CRÍTICO",IF(D29/C29&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F29" s="5" t="n"/>
     </row>
@@ -980,10 +1020,9 @@
       <c r="D30" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>AGOTADO</t>
-        </is>
+      <c r="E30" s="8">
+        <f>IF(D30=0,"AGOTADO",IF(D30/C30&lt;=0.15,"CRÍTICO",IF(D30/C30&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
       </c>
       <c r="F30" s="5" t="n"/>
     </row>
@@ -1087,6 +1126,48 @@
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B32:F32"/>
   </mergeCells>
+  <conditionalFormatting sqref="E7:E12">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"BAJO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"CRÍTICO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"AGOTADO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16:E21">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="0">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="1">
+      <formula>"BAJO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="2">
+      <formula>"CRÍTICO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="3">
+      <formula>"AGOTADO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25:E30">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="0">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="1">
+      <formula>"BAJO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="2">
+      <formula>"CRÍTICO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="3">
+      <formula>"AGOTADO"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1097,20 +1178,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G22"/>
+  <dimension ref="A2:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>HISTORIAL DE INVENTARIO — LOTE 34 MZA 14</t>
         </is>
@@ -1119,437 +1203,587 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>De arriba (inicial / completo) hacia abajo (más reciente)</t>
+          <t>Salió = lo que se sacó del almacén ese día · Queda = saldo restante</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Fecha / Corte</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Pisero(s)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Salió Moret</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Salió Duela</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>Piso Moret</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>Urbania White</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>Malla Lyndhurst</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>Royal Walnut</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>Pegavitro</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>Unicrest</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>▶ Inicial (completo)</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="n">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>▶ Inicial</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr"/>
+      <c r="C6" s="12" t="inlineStr"/>
+      <c r="D6" s="12" t="inlineStr"/>
+      <c r="E6" s="12" t="n">
         <v>117</v>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="D6" s="11" t="n">
+      <c r="F6" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="H6" s="12" t="n">
         <v>41</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="I6" s="12" t="n">
         <v>93</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="J6" s="12" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>30 abr</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Valdez+Joel</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="6" t="n">
         <v>110</v>
       </c>
-      <c r="C7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D7" s="6" t="n">
+      <c r="F7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="H7" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="I7" s="6" t="n">
         <v>84</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="J7" s="6" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>01 may</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Valdez+Orduño</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr"/>
+      <c r="D8" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="6" t="n">
         <v>110</v>
       </c>
-      <c r="C8" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" s="6" t="n">
+      <c r="F8" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="H8" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="I8" s="6" t="n">
         <v>74</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="J8" s="6" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>02 may</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Valdez+Orduño</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr"/>
+      <c r="D9" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="6" t="n">
         <v>110</v>
       </c>
-      <c r="C9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D9" s="6" t="n">
+      <c r="F9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="H9" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="I9" s="6" t="n">
         <v>69</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="J9" s="6" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>05 may</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Valdez+Joel</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="6" t="n">
         <v>105</v>
       </c>
-      <c r="C10" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D10" s="6" t="n">
+      <c r="F10" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G10" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="H10" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="I10" s="6" t="n">
         <v>59</v>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="J10" s="6" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>06 may</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Valdez+Joel</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr"/>
+      <c r="D11" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="6" t="n">
         <v>105</v>
       </c>
-      <c r="C11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D11" s="6" t="n">
+      <c r="F11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G11" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="H11" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="I11" s="6" t="n">
         <v>55</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="J11" s="6" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>07 may</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Gerardo Orduño</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="C12" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D12" s="6" t="n">
+      <c r="F12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G12" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="H12" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="I12" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="J12" s="6" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>08 may</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Gerardo Orduño</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="6" t="n">
         <v>99</v>
       </c>
-      <c r="C13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D13" s="6" t="n">
+      <c r="F13" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="6" t="n">
+      <c r="H13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="J13" s="6" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>11 may</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Gerardo Orduño</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" s="14" t="inlineStr"/>
+      <c r="E14" s="6" t="n">
         <v>94</v>
       </c>
-      <c r="C14" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D14" s="6" t="n">
+      <c r="F14" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G14" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="6" t="n">
+      <c r="H14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="J14" s="6" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>13 may</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Gerardo Orduño</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="14" t="inlineStr"/>
+      <c r="E15" s="6" t="n">
         <v>89</v>
       </c>
-      <c r="C15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D15" s="6" t="n">
+      <c r="F15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G15" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="6" t="n">
+      <c r="H15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="J15" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>15 may</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Gerardo Orduño</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="D16" s="14" t="inlineStr"/>
+      <c r="E16" s="6" t="n">
         <v>82</v>
       </c>
-      <c r="C16" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D16" s="6" t="n">
+      <c r="F16" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="6" t="n">
+      <c r="H16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="J16" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>19 may</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Jaime</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="14" t="inlineStr"/>
+      <c r="E17" s="6" t="n">
         <v>79</v>
       </c>
-      <c r="C17" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D17" s="6" t="n">
+      <c r="F17" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G17" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="6" t="n">
+      <c r="H17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="J17" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>20 may</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Jaime</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr"/>
+      <c r="D18" s="14" t="inlineStr"/>
+      <c r="E18" s="6" t="n">
         <v>79</v>
       </c>
-      <c r="C18" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D18" s="6" t="n">
+      <c r="F18" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G18" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="6" t="n">
+      <c r="H18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="J18" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>22 may</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Jaime</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="D19" s="14" t="inlineStr"/>
+      <c r="E19" s="6" t="n">
         <v>55</v>
       </c>
-      <c r="C19" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D19" s="6" t="n">
+      <c r="F19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G19" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="6" t="n">
+      <c r="H19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="J19" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>1-6 jun (P.B.)</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>1-6 jun</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón (P.B.)</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>51</v>
+      </c>
+      <c r="D20" s="14" t="inlineStr"/>
+      <c r="E20" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="6" t="n">
+      <c r="F20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="E20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="6" t="n">
+      <c r="H20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>15-20 jun (vitroblock)</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>15-20 jun</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>vitroblock 28 pz</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="14" t="inlineStr"/>
       <c r="E21" s="6" t="n">
         <v>0</v>
       </c>
@@ -1559,36 +1793,48 @@
       <c r="G21" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="H21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>★ Corte final (actual)</t>
         </is>
       </c>
-      <c r="B22" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="14" t="n">
+      <c r="B22" s="15" t="inlineStr"/>
+      <c r="C22" s="16" t="inlineStr"/>
+      <c r="D22" s="16" t="inlineStr"/>
+      <c r="E22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="16" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1600,20 +1846,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G12"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>HISTORIAL DE INVENTARIO — LOTE 9 MZA 7</t>
         </is>
@@ -1622,226 +1872,891 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>De arriba (inicial / completo) hacia abajo (más reciente)</t>
-        </is>
-      </c>
-    </row>
+          <t>Salió = lo que se sacó del almacén ese día · Queda = saldo restante</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Fecha / Corte</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Pisero(s)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Salió Moret</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Salió Duela</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>Piso Moret</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>Urbania White</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>Malla Lyndhurst</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>Royal Walnut</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>Pegavitro</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>Fija Porcelánico</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>▶ Inicial (completo)</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="n">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>▶ Inicial</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr"/>
+      <c r="C6" s="12" t="inlineStr"/>
+      <c r="D6" s="12" t="inlineStr"/>
+      <c r="E6" s="12" t="n">
         <v>98</v>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="D6" s="11" t="n">
+      <c r="F6" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="H6" s="12" t="n">
         <v>37</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="I6" s="12" t="n">
         <v>79</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="J6" s="12" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>20 may</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Cortez (Miguel/Manuel/José A.)</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>21 may</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Cortez</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>93</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>22 may</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Cortez</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>91</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>23 may</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D7" s="6" t="n">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Cortez</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>89</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G10" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="E7" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>59</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>30 may</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>82</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" s="6" t="n">
+      <c r="H10" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>24 may</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Cortez</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>86</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G11" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="E8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="G8" s="6" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>06 jun</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>55</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>13 jun</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>20 jun</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>3</v>
+      <c r="H11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>★ Corte final (actual)</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="n">
-        <v>0</v>
+          <t>25 may</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Cortez</t>
+        </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D12" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>26 may</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Cortez</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>01 jun</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Kevin+Josué+JoséC</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="14" t="inlineStr"/>
+      <c r="E14" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>02 jun</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Kevin+Josué</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="14" t="inlineStr"/>
+      <c r="E15" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>03 jun</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Josué</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="14" t="inlineStr"/>
+      <c r="E16" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>04 jun</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Kevin+Josué</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="14" t="inlineStr"/>
+      <c r="E17" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>05 jun</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Kevin+Josué</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" s="14" t="inlineStr"/>
+      <c r="E18" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>06 jun</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Kevin+Josué</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="14" t="inlineStr"/>
+      <c r="E19" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>08 jun</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Kevin+Josué+JoséC</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" s="14" t="inlineStr"/>
+      <c r="E20" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>09 jun</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Kevin+Josué+JoséC</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" s="14" t="inlineStr"/>
+      <c r="E21" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>10 jun</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Kevin+Josué</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="D22" s="14" t="inlineStr"/>
+      <c r="E22" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>12 jun</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Kevin</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D23" s="14" t="inlineStr"/>
+      <c r="E23" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>16 jun</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Kevin</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="14" t="inlineStr"/>
+      <c r="E24" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>17 jun</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Kevin</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="14" t="inlineStr"/>
+      <c r="E25" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>18 jun</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Kevin</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="14" t="inlineStr"/>
+      <c r="E26" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>23 jun</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="14" t="inlineStr"/>
+      <c r="E27" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>24 jun</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" s="14" t="inlineStr"/>
+      <c r="E28" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="E12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="14" t="n">
+      <c r="H28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>★ Corte final</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Salmerón</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" s="16" t="inlineStr"/>
+      <c r="E29" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="H29" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="16" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1853,20 +2768,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G8"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>HISTORIAL DE INVENTARIO — LOTE 10 MZA 7 (ACTIVO)</t>
         </is>
@@ -1875,126 +2794,487 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>De arriba (inicial / completo) hacia abajo (más reciente)</t>
-        </is>
-      </c>
-    </row>
+          <t>Salió = lo que se sacó del almacén ese día · Queda = saldo restante</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Fecha / Corte</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Pisero(s)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Salió Moret</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Salió Duela</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>Piso Moret</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>Urbania White</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>Malla Lyndhurst</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>Royal Walnut</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>Pegavitro</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>Fija Porcelánico</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>▶ Inicial (completo)</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="n">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>▶ Inicial</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr"/>
+      <c r="C6" s="12" t="inlineStr"/>
+      <c r="D6" s="12" t="inlineStr"/>
+      <c r="E6" s="12" t="n">
         <v>98</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="F6" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="G6" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="H6" s="12" t="n">
         <v>37</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="I6" s="12" t="n">
         <v>79</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="J6" s="12" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>20 jun</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>63</v>
-      </c>
-      <c r="C7" s="6" t="n">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>15 jun</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Josué</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="D7" s="6" t="n">
-        <v>13</v>
+      <c r="D7" s="14" t="n">
+        <v>5</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>15</v>
+        <v>91</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>25</v>
+        <v>16</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>★ Actual (al irme)</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>48</v>
+          <t>16 jun</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Josué</t>
+        </is>
       </c>
       <c r="C8" s="14" t="n">
         <v>7</v>
       </c>
       <c r="D8" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>17 jun</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Salmerón+Josué</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>77</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>18 jun</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Josué</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>19 jun</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>entrega a sitio</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>67</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>20 jun</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>entrega a sitio</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>23 jun</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Kevin</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>24 jun</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Kevin</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>25 jun</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>entrega a sitio</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>26 jun</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>entrega a sitio</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="14" t="inlineStr"/>
+      <c r="E16" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>★ Corte final</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>entrega a sitio</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="16" t="inlineStr"/>
+      <c r="E17" s="16" t="n">
+        <v>48</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="G17" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="E8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="14" t="n">
+      <c r="H17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="16" t="n">
         <v>41</v>
       </c>
-      <c r="G8" s="14" t="n">
+      <c r="J17" s="16" t="n">
         <v>14</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Historial: nombres simples de pisero, sin entregas a sitio, L10 a días reales, vitroblock a inventario
- Etiqueta = solo nombre del pisero principal (Jesús Valdez/Jaime/Miguel Cortez/Jesús Salmerón)
- Eliminadas filas 'entrega a sitio'; L10 queda con los días reales de asistencia (15-18, 23-24 jun)
- L10: días de 2 piseros (15-17 jun) mueven más material que los de 1 pisero (regla del dueño)
- Vitroblock 28 pz movido de etiqueta a renglón de inventario (Resumen L34)
- Verificado por council: cierra exacto y no creciente en los 3 lotes

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXSZ5Q2QVHttNZRkf7MNkK
</commit_message>
<xml_diff>
--- a/Viñas Norte - Inventario y Historial (cierre).xlsx
+++ b/Viñas Norte - Inventario y Historial (cierre).xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F39"/>
+  <dimension ref="B2:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -889,66 +889,66 @@
       </c>
       <c r="F21" s="7" t="n"/>
     </row>
-    <row r="23">
-      <c r="B23" s="3" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Vitroblock P.A. (pza)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="6">
+        <f>IF(D22=0,"AGOTADO",IF(D22/C22&lt;=0.15,"CRÍTICO",IF(D22/C22&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
+      </c>
+      <c r="F22" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>📦  LOTE 9 (MERLOT) MZA 7</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Inicial</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Piso Moret</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="n">
-        <v>98</v>
-      </c>
-      <c r="D25" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="6">
-        <f>IF(D25=0,"AGOTADO",IF(D25/C25&lt;=0.15,"CRÍTICO",IF(D25/C25&lt;=0.4,"BAJO","OK")))</f>
-        <v/>
-      </c>
-      <c r="F25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Urbania White</t>
+          <t>Piso Moret</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>8</v>
+        <v>98</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>0</v>
@@ -962,14 +962,14 @@
     <row r="27">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Malla Lyndhurst</t>
+          <t>Urbania White</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E27" s="6">
         <f>IF(D27=0,"AGOTADO",IF(D27/C27&lt;=0.15,"CRÍTICO",IF(D27/C27&lt;=0.4,"BAJO","OK")))</f>
@@ -980,14 +980,14 @@
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Royal Walnut (duela)</t>
+          <t>Malla Lyndhurst</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E28" s="6">
         <f>IF(D28=0,"AGOTADO",IF(D28/C28&lt;=0.15,"CRÍTICO",IF(D28/C28&lt;=0.4,"BAJO","OK")))</f>
@@ -998,11 +998,11 @@
     <row r="29">
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Pegavitro</t>
+          <t>Royal Walnut (duela)</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="D29" s="6" t="n">
         <v>0</v>
@@ -1016,11 +1016,11 @@
     <row r="30">
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Fija Porcelánico</t>
+          <t>Pegavitro</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="D30" s="6" t="n">
         <v>0</v>
@@ -1031,37 +1031,40 @@
       </c>
       <c r="F30" s="7" t="n"/>
     </row>
-    <row r="32">
-      <c r="B32" s="3" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Fija Porcelánico</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="6">
+        <f>IF(D31=0,"AGOTADO",IF(D31/C31&lt;=0.15,"CRÍTICO",IF(D31/C31&lt;=0.4,"BAJO","OK")))</f>
+        <v/>
+      </c>
+      <c r="F31" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>🧰  EXTRAS Y GENERAL · ALMACÉN</t>
         </is>
       </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>Boquilla Crest Cantera 5 kg</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>3 cajas</t>
-        </is>
-      </c>
-      <c r="D33" s="10" t="n"/>
-      <c r="E33" s="10" t="n"/>
-      <c r="F33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Boquilla Crest Blanco 5 kg</t>
+          <t>Boquilla Crest Cantera 5 kg</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>2 cajas</t>
+          <t>3 cajas</t>
         </is>
       </c>
       <c r="D34" s="10" t="n"/>
@@ -1071,7 +1074,7 @@
     <row r="35">
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Boquilla Crest Chocolate 5 kg</t>
+          <t>Boquilla Crest Blanco 5 kg</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
@@ -1086,12 +1089,12 @@
     <row r="36">
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Boquilla Crest Plata 5 kg</t>
+          <t>Boquilla Crest Chocolate 5 kg</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>1 caja</t>
+          <t>2 cajas</t>
         </is>
       </c>
       <c r="D36" s="10" t="n"/>
@@ -1101,12 +1104,12 @@
     <row r="37">
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Kretbond 20 kg (basecoat)</t>
+          <t>Boquilla Crest Plata 5 kg</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>5 sacos</t>
+          <t>1 caja</t>
         </is>
       </c>
       <c r="D37" s="10" t="n"/>
@@ -1116,12 +1119,12 @@
     <row r="38">
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Econotex/Recubritech fino 20 kg</t>
+          <t>Kretbond 20 kg (basecoat)</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>2 sacos</t>
+          <t>5 sacos</t>
         </is>
       </c>
       <c r="D38" s="10" t="n"/>
@@ -1131,26 +1134,41 @@
     <row r="39">
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>BlueFence 20 lt (impermeabilizante)</t>
+          <t>Econotex/Recubritech fino 20 kg</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>1 cubeta</t>
+          <t>2 sacos</t>
         </is>
       </c>
       <c r="D39" s="10" t="n"/>
       <c r="E39" s="10" t="n"/>
       <c r="F39" s="10" t="n"/>
     </row>
+    <row r="40">
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>BlueFence 20 lt (impermeabilizante)</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>1 cubeta</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B24:F24"/>
     <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B33:F33"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B23:F23"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B32:F32"/>
   </mergeCells>
   <conditionalFormatting sqref="E7:E12">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -1166,7 +1184,7 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E16:E21">
+  <conditionalFormatting sqref="E16:E22">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="0">
       <formula>"AGOTADO"</formula>
     </cfRule>
@@ -1180,7 +1198,7 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E25:E30">
+  <conditionalFormatting sqref="E26:E31">
     <cfRule type="cellIs" priority="9" operator="equal" dxfId="0">
       <formula>"AGOTADO"</formula>
     </cfRule>
@@ -1335,7 +1353,7 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Solo Jesús Valdez</t>
+          <t>Jesús Valdez</t>
         </is>
       </c>
       <c r="C7" s="17" t="n">
@@ -1375,7 +1393,7 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Solo Jesús Valdez</t>
+          <t>Jesús Valdez</t>
         </is>
       </c>
       <c r="C8" s="17" t="n"/>
@@ -1413,7 +1431,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Solo Jesús Valdez</t>
+          <t>Jesús Valdez</t>
         </is>
       </c>
       <c r="C9" s="17" t="n"/>
@@ -1451,7 +1469,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Solo Jesús Valdez</t>
+          <t>Jesús Valdez</t>
         </is>
       </c>
       <c r="C10" s="17" t="n">
@@ -1491,7 +1509,7 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>Solo Jesús Valdez</t>
+          <t>Jesús Valdez</t>
         </is>
       </c>
       <c r="C11" s="17" t="n"/>
@@ -1529,7 +1547,7 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>Solo Jesús Valdez</t>
+          <t>Jesús Valdez</t>
         </is>
       </c>
       <c r="C12" s="17" t="n">
@@ -1571,7 +1589,7 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>Solo Jesús Valdez</t>
+          <t>Jesús Valdez</t>
         </is>
       </c>
       <c r="C13" s="17" t="n">
@@ -1613,7 +1631,7 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>Solo Jesús Valdez</t>
+          <t>Jesús Valdez</t>
         </is>
       </c>
       <c r="C14" s="17" t="n">
@@ -1651,7 +1669,7 @@
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>Solo Jesús Valdez</t>
+          <t>Jesús Valdez</t>
         </is>
       </c>
       <c r="C15" s="17" t="n">
@@ -1691,7 +1709,7 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>Solo Jesús Valdez</t>
+          <t>Jesús Valdez</t>
         </is>
       </c>
       <c r="C16" s="17" t="n">
@@ -1731,7 +1749,7 @@
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>Solo Jaime</t>
+          <t>Jaime</t>
         </is>
       </c>
       <c r="C17" s="17" t="n">
@@ -1767,7 +1785,7 @@
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>Solo Jaime</t>
+          <t>Jaime</t>
         </is>
       </c>
       <c r="C18" s="17" t="n"/>
@@ -1803,7 +1821,7 @@
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>Solo Jaime</t>
+          <t>Jaime</t>
         </is>
       </c>
       <c r="C19" s="17" t="n">
@@ -1841,7 +1859,7 @@
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C20" s="17" t="n">
@@ -1861,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="19" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="J20" s="19" t="n">
         <v>0</v>
@@ -1876,12 +1894,12 @@
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>15-20 jun</t>
+          <t>15-27 jun</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón (vitroblock)</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C21" s="17" t="n">
@@ -1954,7 +1972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L29"/>
+  <dimension ref="A2:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2085,7 +2103,7 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Solo Miguel Cortez</t>
+          <t>Miguel Cortez</t>
         </is>
       </c>
       <c r="C7" s="17" t="n">
@@ -2127,7 +2145,7 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Solo Miguel Cortez</t>
+          <t>Miguel Cortez</t>
         </is>
       </c>
       <c r="C8" s="17" t="n">
@@ -2169,7 +2187,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Solo Miguel Cortez</t>
+          <t>Miguel Cortez</t>
         </is>
       </c>
       <c r="C9" s="17" t="n">
@@ -2211,7 +2229,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Solo Miguel Cortez</t>
+          <t>Miguel Cortez</t>
         </is>
       </c>
       <c r="C10" s="17" t="n">
@@ -2253,7 +2271,7 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>Solo Miguel Cortez</t>
+          <t>Miguel Cortez</t>
         </is>
       </c>
       <c r="C11" s="17" t="n">
@@ -2295,7 +2313,7 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>Solo Miguel Cortez</t>
+          <t>Miguel Cortez</t>
         </is>
       </c>
       <c r="C12" s="17" t="n">
@@ -2337,7 +2355,7 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>Solo Miguel Cortez</t>
+          <t>Miguel Cortez</t>
         </is>
       </c>
       <c r="C13" s="17" t="n">
@@ -2379,7 +2397,7 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C14" s="17" t="n">
@@ -2417,7 +2435,7 @@
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C15" s="17" t="n">
@@ -2455,7 +2473,7 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C16" s="17" t="n">
@@ -2493,7 +2511,7 @@
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C17" s="17" t="n">
@@ -2531,7 +2549,7 @@
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C18" s="17" t="n">
@@ -2569,7 +2587,7 @@
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C19" s="17" t="n">
@@ -2607,7 +2625,7 @@
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C20" s="17" t="n">
@@ -2647,7 +2665,7 @@
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C21" s="17" t="n">
@@ -2687,7 +2705,7 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C22" s="17" t="n">
@@ -2727,7 +2745,7 @@
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C23" s="17" t="n">
@@ -2767,7 +2785,7 @@
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C24" s="17" t="n">
@@ -2807,7 +2825,7 @@
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C25" s="17" t="n">
@@ -2847,7 +2865,7 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C26" s="17" t="n">
@@ -2887,7 +2905,7 @@
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C27" s="17" t="n">
@@ -2927,7 +2945,7 @@
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C28" s="17" t="n">
@@ -2962,40 +2980,78 @@
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>★ Corte final</t>
+          <t>26 jun</t>
         </is>
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" s="17" t="n"/>
       <c r="E29" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F29" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="20" t="n">
+      <c r="G29" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="J29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" s="20" t="n">
+      <c r="J29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" s="19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>★ Corte final</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>Jesús Salmerón</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="17" t="n"/>
+      <c r="E30" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="17" t="n"/>
+      <c r="G30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="J30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3014,7 +3070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L17"/>
+  <dimension ref="A2:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3145,38 +3201,38 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C7" s="17" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D7" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" s="17" t="n">
-        <v>2</v>
-      </c>
       <c r="G7" s="19" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H7" s="19" t="n">
         <v>7</v>
       </c>
       <c r="I7" s="19" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J7" s="19" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="L7" s="19" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
@@ -3187,38 +3243,38 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D8" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8" s="17" t="n">
-        <v>3</v>
-      </c>
       <c r="G8" s="19" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="H8" s="19" t="n">
         <v>7</v>
       </c>
       <c r="I8" s="19" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J8" s="19" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="L8" s="19" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -3229,38 +3285,38 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C9" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="17" t="n">
-        <v>5</v>
-      </c>
       <c r="E9" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="17" t="n">
-        <v>2</v>
-      </c>
       <c r="G9" s="19" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="H9" s="19" t="n">
         <v>7</v>
       </c>
       <c r="I9" s="19" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J9" s="19" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="L9" s="19" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -3271,95 +3327,95 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Solo Salmerón</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C10" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="D10" s="17" t="n">
-        <v>5</v>
-      </c>
       <c r="E10" s="17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="H10" s="19" t="n">
         <v>7</v>
       </c>
       <c r="I10" s="19" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J10" s="19" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="L10" s="19" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>19 jun</t>
+          <t>23 jun</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>entrega a sitio</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C11" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D11" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="D11" s="17" t="n">
+      <c r="E11" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="17" t="n">
-        <v>3</v>
-      </c>
       <c r="F11" s="17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="H11" s="19" t="n">
         <v>7</v>
       </c>
       <c r="I11" s="19" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J11" s="19" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="L11" s="19" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>20 jun</t>
+          <t>★ 24 jun (saldo actual)</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>entrega a sitio</t>
+          <t>Jesús Salmerón</t>
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D12" s="17" t="n">
         <v>4</v>
@@ -3368,230 +3424,24 @@
         <v>4</v>
       </c>
       <c r="F12" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G12" s="19" t="n">
-        <v>63</v>
-      </c>
-      <c r="H12" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="H12" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="I12" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="J12" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="K12" s="19" t="n">
-        <v>58</v>
-      </c>
-      <c r="L12" s="19" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>23 jun</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>Solo Salmerón</t>
-        </is>
-      </c>
-      <c r="C13" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="19" t="n">
-        <v>60</v>
-      </c>
-      <c r="H13" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="J13" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="K13" s="19" t="n">
-        <v>55</v>
-      </c>
-      <c r="L13" s="19" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>24 jun</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>Solo Salmerón</t>
-        </is>
-      </c>
-      <c r="C14" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D14" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="E14" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F14" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G14" s="19" t="n">
-        <v>57</v>
-      </c>
-      <c r="H14" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="I14" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="J14" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K14" s="19" t="n">
-        <v>51</v>
-      </c>
-      <c r="L14" s="19" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>25 jun</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>entrega a sitio</t>
-        </is>
-      </c>
-      <c r="C15" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D15" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="F15" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="G15" s="19" t="n">
-        <v>54</v>
-      </c>
-      <c r="H15" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="I15" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="J15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="19" t="n">
-        <v>48</v>
-      </c>
-      <c r="L15" s="19" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>26 jun</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>entrega a sitio</t>
-        </is>
-      </c>
-      <c r="C16" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F16" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" s="19" t="n">
-        <v>51</v>
-      </c>
-      <c r="H16" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="I16" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="J16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="19" t="n">
-        <v>44</v>
-      </c>
-      <c r="L16" s="19" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>★ Corte final</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>entrega a sitio</t>
-        </is>
-      </c>
-      <c r="C17" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D17" s="17" t="n"/>
-      <c r="E17" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="F17" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" s="20" t="n">
-        <v>48</v>
-      </c>
-      <c r="H17" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="I17" s="20" t="n">
+      <c r="I12" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="J17" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="20" t="n">
+      <c r="J12" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="L17" s="20" t="n">
+      <c r="L12" s="20" t="n">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Historial: columnas Salió Urbania/Malla por día + recalc de Estado al abrir
- Nuevas columnas Salió Urbania y Salió Malla (delta diario), con timing anclado a los destajos de baño/charola/sardinel/nichos
- L34: charolas en semanas de baño (Valdez may, Jaime 19-22 may, Salmerón P.B. jun)
- L9: charolas repartidas entre baño Cortez (may) y baños P.A. Salmerón (jun)
- L10: charolas concentradas 23-24 jun (semana de baños/sardinel/nichos)
- Estado: fullCalcOnLoad=True para que 'AGOTADO' se calcule al abrir (ya no sale en blanco)
- Council: L34/L9 aprobados; L10 corregido (Malla)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXSZ5Q2QVHttNZRkf7MNkK
</commit_message>
<xml_diff>
--- a/Viñas Norte - Inventario y Historial (cierre).xlsx
+++ b/Viñas Norte - Inventario y Historial (cierre).xlsx
@@ -1222,7 +1222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L22"/>
+  <dimension ref="A2:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1237,6 +1237,8 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1271,45 +1273,55 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
+          <t>Salió Urbania</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Salió Malla</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
           <t>Salió Duela</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Salió Pegavitro</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>Salió Unicrest</t>
         </is>
       </c>
-      <c r="G5" s="13" t="inlineStr">
+      <c r="I5" s="13" t="inlineStr">
         <is>
           <t>Piso Moret</t>
         </is>
       </c>
-      <c r="H5" s="13" t="inlineStr">
+      <c r="J5" s="13" t="inlineStr">
         <is>
           <t>Urbania White</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>Malla Lyndhurst</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="L5" s="13" t="inlineStr">
         <is>
           <t>Royal Walnut</t>
         </is>
       </c>
-      <c r="K5" s="13" t="inlineStr">
+      <c r="M5" s="13" t="inlineStr">
         <is>
           <t>Pegavitro</t>
         </is>
       </c>
-      <c r="L5" s="13" t="inlineStr">
+      <c r="N5" s="13" t="inlineStr">
         <is>
           <t>Unicrest</t>
         </is>
@@ -1326,22 +1338,24 @@
       <c r="D6" s="17" t="n"/>
       <c r="E6" s="17" t="n"/>
       <c r="F6" s="17" t="n"/>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="17" t="n"/>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="18" t="n">
         <v>117</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="J6" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="K6" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="L6" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="M6" s="18" t="n">
         <v>93</v>
       </c>
-      <c r="L6" s="18" t="n">
+      <c r="N6" s="18" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1359,29 +1373,31 @@
       <c r="C7" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="G7" s="17" t="n">
         <v>9</v>
       </c>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="19" t="n">
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="19" t="n">
         <v>110</v>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="J7" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="K7" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="L7" s="19" t="n">
         <v>36</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="M7" s="19" t="n">
         <v>84</v>
       </c>
-      <c r="L7" s="19" t="n">
+      <c r="N7" s="19" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1397,29 +1413,31 @@
         </is>
       </c>
       <c r="C8" s="17" t="n"/>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="G8" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="F8" s="17" t="n"/>
-      <c r="G8" s="19" t="n">
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="19" t="n">
         <v>110</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="J8" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="K8" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="L8" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="M8" s="19" t="n">
         <v>74</v>
       </c>
-      <c r="L8" s="19" t="n">
+      <c r="N8" s="19" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1435,29 +1453,31 @@
         </is>
       </c>
       <c r="C9" s="17" t="n"/>
-      <c r="D9" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="17" t="n">
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
+      <c r="F9" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="17" t="n"/>
-      <c r="G9" s="19" t="n">
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="19" t="n">
         <v>110</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="J9" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="K9" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="L9" s="19" t="n">
         <v>22</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="M9" s="19" t="n">
         <v>69</v>
       </c>
-      <c r="L9" s="19" t="n">
+      <c r="N9" s="19" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1475,29 +1495,31 @@
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="G10" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="F10" s="17" t="n"/>
-      <c r="G10" s="19" t="n">
+      <c r="H10" s="17" t="n"/>
+      <c r="I10" s="19" t="n">
         <v>105</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="J10" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="K10" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="L10" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="M10" s="19" t="n">
         <v>59</v>
       </c>
-      <c r="L10" s="19" t="n">
+      <c r="N10" s="19" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1513,29 +1535,31 @@
         </is>
       </c>
       <c r="C11" s="17" t="n"/>
-      <c r="D11" s="17" t="n">
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="17" t="n"/>
+      <c r="F11" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F11" s="17" t="n"/>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="19" t="n">
         <v>105</v>
       </c>
-      <c r="H11" s="19" t="n">
+      <c r="J11" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I11" s="19" t="n">
+      <c r="K11" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="L11" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="M11" s="19" t="n">
         <v>55</v>
       </c>
-      <c r="L11" s="19" t="n">
+      <c r="N11" s="19" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1553,31 +1577,33 @@
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="G12" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="F12" s="17" t="n">
+      <c r="H12" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="19" t="n">
+      <c r="I12" s="19" t="n">
         <v>100</v>
       </c>
-      <c r="H12" s="19" t="n">
+      <c r="J12" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="K12" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="J12" s="19" t="n">
+      <c r="L12" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="K12" s="19" t="n">
+      <c r="M12" s="19" t="n">
         <v>45</v>
       </c>
-      <c r="L12" s="19" t="n">
+      <c r="N12" s="19" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1595,31 +1621,35 @@
       <c r="C13" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="17" t="n">
         <v>2</v>
-      </c>
-      <c r="E13" s="17" t="n">
-        <v>4</v>
       </c>
       <c r="F13" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="19" t="n">
+      <c r="G13" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="19" t="n">
         <v>99</v>
       </c>
-      <c r="H13" s="19" t="n">
+      <c r="J13" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I13" s="19" t="n">
-        <v>28</v>
-      </c>
-      <c r="J13" s="19" t="n">
-        <v>0</v>
-      </c>
       <c r="K13" s="19" t="n">
+        <v>26</v>
+      </c>
+      <c r="L13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="19" t="n">
         <v>41</v>
       </c>
-      <c r="L13" s="19" t="n">
+      <c r="N13" s="19" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1637,27 +1667,33 @@
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="17" t="n"/>
-      <c r="F14" s="17" t="n">
+      <c r="D14" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="17" t="n"/>
+      <c r="H14" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="G14" s="19" t="n">
+      <c r="I14" s="19" t="n">
         <v>94</v>
       </c>
-      <c r="H14" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I14" s="19" t="n">
-        <v>28</v>
-      </c>
       <c r="J14" s="19" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K14" s="19" t="n">
+        <v>24</v>
+      </c>
+      <c r="L14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="19" t="n">
         <v>41</v>
       </c>
-      <c r="L14" s="19" t="n">
+      <c r="N14" s="19" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1675,29 +1711,35 @@
       <c r="C15" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="17" t="n"/>
+      <c r="D15" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="E15" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="F15" s="17" t="n">
+      <c r="H15" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="19" t="n">
+      <c r="I15" s="19" t="n">
         <v>89</v>
       </c>
-      <c r="H15" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I15" s="19" t="n">
-        <v>28</v>
-      </c>
       <c r="J15" s="19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K15" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="L15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="19" t="n">
         <v>36</v>
       </c>
-      <c r="L15" s="19" t="n">
+      <c r="N15" s="19" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1716,28 +1758,30 @@
         <v>7</v>
       </c>
       <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="17" t="n">
+      <c r="H16" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="19" t="n">
+      <c r="I16" s="19" t="n">
         <v>82</v>
       </c>
-      <c r="H16" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I16" s="19" t="n">
-        <v>28</v>
-      </c>
       <c r="J16" s="19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K16" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="L16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="19" t="n">
         <v>34</v>
       </c>
-      <c r="L16" s="19" t="n">
+      <c r="N16" s="19" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1755,25 +1799,31 @@
       <c r="C17" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="D17" s="17" t="n"/>
-      <c r="E17" s="17" t="n"/>
+      <c r="D17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>4</v>
+      </c>
       <c r="F17" s="17" t="n"/>
-      <c r="G17" s="19" t="n">
+      <c r="G17" s="17" t="n"/>
+      <c r="H17" s="17" t="n"/>
+      <c r="I17" s="19" t="n">
         <v>79</v>
       </c>
-      <c r="H17" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>28</v>
-      </c>
       <c r="J17" s="19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K17" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="L17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="19" t="n">
         <v>34</v>
       </c>
-      <c r="L17" s="19" t="n">
+      <c r="N17" s="19" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1789,27 +1839,33 @@
         </is>
       </c>
       <c r="C18" s="17" t="n"/>
-      <c r="D18" s="17" t="n"/>
+      <c r="D18" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="E18" s="17" t="n">
         <v>4</v>
       </c>
       <c r="F18" s="17" t="n"/>
-      <c r="G18" s="19" t="n">
+      <c r="G18" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H18" s="17" t="n"/>
+      <c r="I18" s="19" t="n">
         <v>79</v>
       </c>
-      <c r="H18" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <v>28</v>
-      </c>
       <c r="J18" s="19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K18" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="L18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="L18" s="19" t="n">
+      <c r="N18" s="19" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1827,27 +1883,33 @@
       <c r="C19" s="17" t="n">
         <v>24</v>
       </c>
-      <c r="D19" s="17" t="n"/>
+      <c r="D19" s="17" t="n">
+        <v>2</v>
+      </c>
       <c r="E19" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="F19" s="17" t="n"/>
+      <c r="G19" s="17" t="n">
         <v>20</v>
       </c>
-      <c r="F19" s="17" t="n"/>
-      <c r="G19" s="19" t="n">
+      <c r="H19" s="17" t="n"/>
+      <c r="I19" s="19" t="n">
         <v>55</v>
       </c>
-      <c r="H19" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I19" s="19" t="n">
-        <v>28</v>
-      </c>
       <c r="J19" s="19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K19" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="L19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L19" s="19" t="n">
+      <c r="N19" s="19" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1865,21 +1927,21 @@
       <c r="C20" s="17" t="n">
         <v>51</v>
       </c>
-      <c r="D20" s="17" t="n"/>
+      <c r="D20" s="17" t="n">
+        <v>2</v>
+      </c>
       <c r="E20" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F20" s="17" t="n"/>
+      <c r="G20" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="F20" s="17" t="n">
+      <c r="H20" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="H20" s="19" t="n">
-        <v>0</v>
-      </c>
       <c r="I20" s="19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J20" s="19" t="n">
         <v>0</v>
@@ -1888,6 +1950,12 @@
         <v>0</v>
       </c>
       <c r="L20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1908,12 +1976,8 @@
       <c r="D21" s="17" t="n"/>
       <c r="E21" s="17" t="n"/>
       <c r="F21" s="17" t="n"/>
-      <c r="G21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="19" t="n">
-        <v>0</v>
-      </c>
+      <c r="G21" s="17" t="n"/>
+      <c r="H21" s="17" t="n"/>
       <c r="I21" s="19" t="n">
         <v>0</v>
       </c>
@@ -1924,6 +1988,12 @@
         <v>0</v>
       </c>
       <c r="L21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1938,12 +2008,8 @@
       <c r="D22" s="17" t="n"/>
       <c r="E22" s="17" t="n"/>
       <c r="F22" s="17" t="n"/>
-      <c r="G22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="20" t="n">
-        <v>0</v>
-      </c>
+      <c r="G22" s="17" t="n"/>
+      <c r="H22" s="17" t="n"/>
       <c r="I22" s="20" t="n">
         <v>0</v>
       </c>
@@ -1954,13 +2020,19 @@
         <v>0</v>
       </c>
       <c r="L22" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="20" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A2:N2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1972,7 +2044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L30"/>
+  <dimension ref="A2:N30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1987,6 +2059,8 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -2021,45 +2095,55 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
+          <t>Salió Urbania</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Salió Malla</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
           <t>Salió Duela</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Salió Pegavitro</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>Salió Porcelánico</t>
         </is>
       </c>
-      <c r="G5" s="13" t="inlineStr">
+      <c r="I5" s="13" t="inlineStr">
         <is>
           <t>Piso Moret</t>
         </is>
       </c>
-      <c r="H5" s="13" t="inlineStr">
+      <c r="J5" s="13" t="inlineStr">
         <is>
           <t>Urbania White</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>Malla Lyndhurst</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="L5" s="13" t="inlineStr">
         <is>
           <t>Royal Walnut</t>
         </is>
       </c>
-      <c r="K5" s="13" t="inlineStr">
+      <c r="M5" s="13" t="inlineStr">
         <is>
           <t>Pegavitro</t>
         </is>
       </c>
-      <c r="L5" s="13" t="inlineStr">
+      <c r="N5" s="13" t="inlineStr">
         <is>
           <t>Fija Porcelánico</t>
         </is>
@@ -2076,22 +2160,24 @@
       <c r="D6" s="17" t="n"/>
       <c r="E6" s="17" t="n"/>
       <c r="F6" s="17" t="n"/>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="17" t="n"/>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="18" t="n">
         <v>98</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="J6" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="K6" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="L6" s="18" t="n">
         <v>37</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="M6" s="18" t="n">
         <v>79</v>
       </c>
-      <c r="L6" s="18" t="n">
+      <c r="N6" s="18" t="n">
         <v>39</v>
       </c>
     </row>
@@ -2109,31 +2195,33 @@
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="G7" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="17" t="n">
+      <c r="H7" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="I7" s="19" t="n">
         <v>96</v>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="J7" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="K7" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="L7" s="19" t="n">
         <v>32</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="M7" s="19" t="n">
         <v>74</v>
       </c>
-      <c r="L7" s="19" t="n">
+      <c r="N7" s="19" t="n">
         <v>36</v>
       </c>
     </row>
@@ -2151,31 +2239,33 @@
       <c r="C8" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="G8" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="17" t="n">
+      <c r="H8" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="I8" s="19" t="n">
         <v>94</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="J8" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="K8" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="L8" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="M8" s="19" t="n">
         <v>69</v>
       </c>
-      <c r="L8" s="19" t="n">
+      <c r="N8" s="19" t="n">
         <v>33</v>
       </c>
     </row>
@@ -2193,31 +2283,33 @@
       <c r="C9" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="17" t="n">
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
+      <c r="F9" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="17" t="n">
+      <c r="H9" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="I9" s="19" t="n">
         <v>93</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="J9" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="K9" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="L9" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="M9" s="19" t="n">
         <v>64</v>
       </c>
-      <c r="L9" s="19" t="n">
+      <c r="N9" s="19" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2235,31 +2327,33 @@
       <c r="C10" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="G10" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="F10" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="19" t="n">
+      <c r="H10" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" s="19" t="n">
         <v>89</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="J10" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="K10" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="L10" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="M10" s="19" t="n">
         <v>57</v>
       </c>
-      <c r="L10" s="19" t="n">
+      <c r="N10" s="19" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2277,31 +2371,35 @@
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="D11" s="17" t="n">
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="17" t="n">
         <v>9</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="G11" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="F11" s="17" t="n">
+      <c r="H11" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="I11" s="19" t="n">
         <v>84</v>
       </c>
-      <c r="H11" s="19" t="n">
+      <c r="J11" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I11" s="19" t="n">
-        <v>17</v>
-      </c>
-      <c r="J11" s="19" t="n">
+      <c r="K11" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="L11" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="M11" s="19" t="n">
         <v>49</v>
       </c>
-      <c r="L11" s="19" t="n">
+      <c r="N11" s="19" t="n">
         <v>22</v>
       </c>
     </row>
@@ -2320,30 +2418,34 @@
         <v>1</v>
       </c>
       <c r="D12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="G12" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="F12" s="17" t="n">
+      <c r="H12" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="19" t="n">
+      <c r="I12" s="19" t="n">
         <v>83</v>
       </c>
-      <c r="H12" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I12" s="19" t="n">
-        <v>17</v>
-      </c>
       <c r="J12" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="K12" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="L12" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="K12" s="19" t="n">
+      <c r="M12" s="19" t="n">
         <v>44</v>
       </c>
-      <c r="L12" s="19" t="n">
+      <c r="N12" s="19" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2361,31 +2463,35 @@
       <c r="C13" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="G13" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="F13" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="19" t="n">
+      <c r="H13" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="19" t="n">
         <v>82</v>
       </c>
-      <c r="H13" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>17</v>
-      </c>
       <c r="J13" s="19" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K13" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="L13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="L13" s="19" t="n">
+      <c r="N13" s="19" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2405,25 +2511,27 @@
       </c>
       <c r="D14" s="17" t="n"/>
       <c r="E14" s="17" t="n"/>
-      <c r="F14" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="19" t="n">
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="17" t="n"/>
+      <c r="H14" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="19" t="n">
         <v>76</v>
       </c>
-      <c r="H14" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I14" s="19" t="n">
-        <v>17</v>
-      </c>
       <c r="J14" s="19" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K14" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="L14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="L14" s="19" t="n">
+      <c r="N14" s="19" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2443,25 +2551,27 @@
       </c>
       <c r="D15" s="17" t="n"/>
       <c r="E15" s="17" t="n"/>
-      <c r="F15" s="17" t="n">
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="17" t="n"/>
+      <c r="H15" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="19" t="n">
+      <c r="I15" s="19" t="n">
         <v>71</v>
       </c>
-      <c r="H15" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I15" s="19" t="n">
-        <v>17</v>
-      </c>
       <c r="J15" s="19" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K15" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="L15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="L15" s="19" t="n">
+      <c r="N15" s="19" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2481,25 +2591,27 @@
       </c>
       <c r="D16" s="17" t="n"/>
       <c r="E16" s="17" t="n"/>
-      <c r="F16" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="19" t="n">
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
+      <c r="H16" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="19" t="n">
         <v>68</v>
       </c>
-      <c r="H16" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I16" s="19" t="n">
-        <v>17</v>
-      </c>
       <c r="J16" s="19" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K16" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="L16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="L16" s="19" t="n">
+      <c r="N16" s="19" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2519,25 +2631,27 @@
       </c>
       <c r="D17" s="17" t="n"/>
       <c r="E17" s="17" t="n"/>
-      <c r="F17" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="19" t="n">
+      <c r="F17" s="17" t="n"/>
+      <c r="G17" s="17" t="n"/>
+      <c r="H17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="19" t="n">
         <v>64</v>
       </c>
-      <c r="H17" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>17</v>
-      </c>
       <c r="J17" s="19" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K17" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="L17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="L17" s="19" t="n">
+      <c r="N17" s="19" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2557,25 +2671,27 @@
       </c>
       <c r="D18" s="17" t="n"/>
       <c r="E18" s="17" t="n"/>
-      <c r="F18" s="17" t="n">
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="17" t="n"/>
+      <c r="H18" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="19" t="n">
+      <c r="I18" s="19" t="n">
         <v>59</v>
       </c>
-      <c r="H18" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <v>17</v>
-      </c>
       <c r="J18" s="19" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K18" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="L18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="L18" s="19" t="n">
+      <c r="N18" s="19" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2595,25 +2711,27 @@
       </c>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
-      <c r="F19" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" s="19" t="n">
+      <c r="F19" s="17" t="n"/>
+      <c r="G19" s="17" t="n"/>
+      <c r="H19" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="19" t="n">
         <v>55</v>
       </c>
-      <c r="H19" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I19" s="19" t="n">
-        <v>17</v>
-      </c>
       <c r="J19" s="19" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K19" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="L19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="L19" s="19" t="n">
+      <c r="N19" s="19" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2632,28 +2750,30 @@
         <v>10</v>
       </c>
       <c r="D20" s="17" t="n"/>
-      <c r="E20" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F20" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="19" t="n">
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
+      <c r="G20" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="19" t="n">
         <v>45</v>
       </c>
-      <c r="H20" s="19" t="n">
+      <c r="J20" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="I20" s="19" t="n">
-        <v>17</v>
-      </c>
-      <c r="J20" s="19" t="n">
-        <v>0</v>
-      </c>
       <c r="K20" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="L20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="19" t="n">
         <v>35</v>
       </c>
-      <c r="L20" s="19" t="n">
+      <c r="N20" s="19" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2671,29 +2791,33 @@
       <c r="C21" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="D21" s="17" t="n"/>
-      <c r="E21" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F21" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="19" t="n">
+      <c r="D21" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="17" t="n"/>
+      <c r="F21" s="17" t="n"/>
+      <c r="G21" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="19" t="n">
         <v>35</v>
       </c>
-      <c r="H21" s="19" t="n">
+      <c r="J21" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="I21" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="J21" s="19" t="n">
-        <v>0</v>
-      </c>
       <c r="K21" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="L21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="L21" s="19" t="n">
+      <c r="N21" s="19" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2713,27 +2837,31 @@
       </c>
       <c r="D22" s="17" t="n"/>
       <c r="E22" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F22" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H22" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="H22" s="19" t="n">
+      <c r="J22" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="I22" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="J22" s="19" t="n">
-        <v>0</v>
-      </c>
       <c r="K22" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="L22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="L22" s="19" t="n">
+      <c r="N22" s="19" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2751,29 +2879,33 @@
       <c r="C23" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="D23" s="17" t="n"/>
-      <c r="E23" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F23" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="19" t="n">
+      <c r="D23" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="17" t="n"/>
+      <c r="F23" s="17" t="n"/>
+      <c r="G23" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="19" t="n">
         <v>21</v>
       </c>
-      <c r="H23" s="19" t="n">
+      <c r="J23" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="I23" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="J23" s="19" t="n">
-        <v>0</v>
-      </c>
       <c r="K23" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="L23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="L23" s="19" t="n">
+      <c r="N23" s="19" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2791,29 +2923,33 @@
       <c r="C24" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="D24" s="17" t="n"/>
-      <c r="E24" s="17" t="n">
+      <c r="D24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="17" t="n"/>
+      <c r="G24" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="F24" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="19" t="n">
+      <c r="H24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="19" t="n">
         <v>18</v>
       </c>
-      <c r="H24" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="I24" s="19" t="n">
-        <v>15</v>
-      </c>
       <c r="J24" s="19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K24" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="L24" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="L24" s="19" t="n">
+      <c r="N24" s="19" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2831,29 +2967,33 @@
       <c r="C25" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="D25" s="17" t="n"/>
-      <c r="E25" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F25" s="17" t="n">
+      <c r="D25" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="17" t="n"/>
+      <c r="F25" s="17" t="n"/>
+      <c r="G25" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" s="17" t="n">
         <v>2</v>
-      </c>
-      <c r="G25" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="H25" s="19" t="n">
-        <v>3</v>
       </c>
       <c r="I25" s="19" t="n">
         <v>15</v>
       </c>
       <c r="J25" s="19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K25" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="L25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="L25" s="19" t="n">
+      <c r="N25" s="19" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2871,29 +3011,35 @@
       <c r="C26" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="D26" s="17" t="n"/>
+      <c r="D26" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="E26" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F26" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="17" t="n"/>
+      <c r="G26" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="H26" s="19" t="n">
+      <c r="J26" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="I26" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="J26" s="19" t="n">
-        <v>0</v>
-      </c>
       <c r="K26" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="L26" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="L26" s="19" t="n">
+      <c r="N26" s="19" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2912,28 +3058,30 @@
         <v>4</v>
       </c>
       <c r="D27" s="17" t="n"/>
-      <c r="E27" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F27" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="19" t="n">
+      <c r="E27" s="17" t="n"/>
+      <c r="F27" s="17" t="n"/>
+      <c r="G27" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H27" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="H27" s="19" t="n">
+      <c r="J27" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="I27" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="J27" s="19" t="n">
-        <v>0</v>
-      </c>
       <c r="K27" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="L27" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="L27" s="19" t="n">
+      <c r="N27" s="19" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2951,29 +3099,33 @@
       <c r="C28" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="D28" s="17" t="n"/>
-      <c r="E28" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F28" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="H28" s="19" t="n">
+      <c r="D28" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="17" t="n"/>
+      <c r="F28" s="17" t="n"/>
+      <c r="G28" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" s="17" t="n">
         <v>1</v>
       </c>
       <c r="I28" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J28" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="J28" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" s="19" t="n">
-        <v>4</v>
-      </c>
       <c r="L28" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="N28" s="19" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2991,29 +3143,33 @@
       <c r="C29" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="D29" s="17" t="n"/>
-      <c r="E29" s="17" t="n">
+      <c r="D29" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="17" t="n"/>
+      <c r="F29" s="17" t="n"/>
+      <c r="G29" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="F29" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H29" s="19" t="n">
-        <v>0</v>
+      <c r="H29" s="17" t="n">
+        <v>1</v>
       </c>
       <c r="I29" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="J29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" s="19" t="n">
-        <v>1</v>
-      </c>
       <c r="L29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N29" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3032,33 +3188,35 @@
         <v>1</v>
       </c>
       <c r="D30" s="17" t="n"/>
-      <c r="E30" s="17" t="n">
-        <v>1</v>
-      </c>
+      <c r="E30" s="17" t="n"/>
       <c r="F30" s="17" t="n"/>
-      <c r="G30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="20" t="n">
-        <v>0</v>
-      </c>
+      <c r="G30" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="17" t="n"/>
       <c r="I30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="J30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="20" t="n">
-        <v>0</v>
-      </c>
       <c r="L30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="20" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A2:N2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3070,7 +3228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L12"/>
+  <dimension ref="A2:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3085,6 +3243,8 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -3119,45 +3279,55 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
+          <t>Salió Urbania</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Salió Malla</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
           <t>Salió Duela</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Salió Pegavitro</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>Salió Porcelánico</t>
         </is>
       </c>
-      <c r="G5" s="13" t="inlineStr">
+      <c r="I5" s="13" t="inlineStr">
         <is>
           <t>Piso Moret</t>
         </is>
       </c>
-      <c r="H5" s="13" t="inlineStr">
+      <c r="J5" s="13" t="inlineStr">
         <is>
           <t>Urbania White</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>Malla Lyndhurst</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="L5" s="13" t="inlineStr">
         <is>
           <t>Royal Walnut</t>
         </is>
       </c>
-      <c r="K5" s="13" t="inlineStr">
+      <c r="M5" s="13" t="inlineStr">
         <is>
           <t>Pegavitro</t>
         </is>
       </c>
-      <c r="L5" s="13" t="inlineStr">
+      <c r="N5" s="13" t="inlineStr">
         <is>
           <t>Fija Porcelánico</t>
         </is>
@@ -3174,22 +3344,24 @@
       <c r="D6" s="17" t="n"/>
       <c r="E6" s="17" t="n"/>
       <c r="F6" s="17" t="n"/>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="17" t="n"/>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="18" t="n">
         <v>98</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="J6" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="K6" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="L6" s="18" t="n">
         <v>37</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="M6" s="18" t="n">
         <v>79</v>
       </c>
-      <c r="L6" s="18" t="n">
+      <c r="N6" s="18" t="n">
         <v>39</v>
       </c>
     </row>
@@ -3207,31 +3379,33 @@
       <c r="C7" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="G7" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="F7" s="17" t="n">
+      <c r="H7" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="I7" s="19" t="n">
         <v>88</v>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="J7" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="I7" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="J7" s="19" t="n">
+      <c r="K7" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="L7" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="M7" s="19" t="n">
         <v>71</v>
       </c>
-      <c r="L7" s="19" t="n">
+      <c r="N7" s="19" t="n">
         <v>34</v>
       </c>
     </row>
@@ -3249,31 +3423,33 @@
       <c r="C8" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="G8" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="F8" s="17" t="n">
+      <c r="H8" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="I8" s="19" t="n">
         <v>78</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="J8" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="I8" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="J8" s="19" t="n">
+      <c r="K8" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="L8" s="19" t="n">
         <v>21</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="M8" s="19" t="n">
         <v>63</v>
       </c>
-      <c r="L8" s="19" t="n">
+      <c r="N8" s="19" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3291,31 +3467,33 @@
       <c r="C9" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
+      <c r="F9" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="G9" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="F9" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="G9" s="19" t="n">
+      <c r="H9" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" s="19" t="n">
         <v>68</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="J9" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="I9" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="J9" s="19" t="n">
+      <c r="K9" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="L9" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="M9" s="19" t="n">
         <v>56</v>
       </c>
-      <c r="L9" s="19" t="n">
+      <c r="N9" s="19" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3333,31 +3511,33 @@
       <c r="C10" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="G10" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="F10" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="19" t="n">
+      <c r="H10" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" s="19" t="n">
         <v>60</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="J10" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="I10" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="J10" s="19" t="n">
+      <c r="K10" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="L10" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="M10" s="19" t="n">
         <v>50</v>
       </c>
-      <c r="L10" s="19" t="n">
+      <c r="N10" s="19" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3375,31 +3555,35 @@
       <c r="C11" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="D11" s="17" t="n">
-        <v>4</v>
-      </c>
+      <c r="D11" s="17" t="n"/>
       <c r="E11" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="F11" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="G11" s="19" t="n">
+      <c r="H11" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" s="19" t="n">
         <v>54</v>
       </c>
-      <c r="H11" s="19" t="n">
+      <c r="J11" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="I11" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="J11" s="19" t="n">
-        <v>4</v>
-      </c>
       <c r="K11" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="L11" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="M11" s="19" t="n">
         <v>45</v>
       </c>
-      <c r="L11" s="19" t="n">
+      <c r="N11" s="19" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3417,38 +3601,42 @@
       <c r="C12" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="D12" s="17" t="n">
-        <v>4</v>
-      </c>
+      <c r="D12" s="17" t="n"/>
       <c r="E12" s="17" t="n">
         <v>4</v>
       </c>
       <c r="F12" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="G12" s="20" t="n">
+      <c r="I12" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="H12" s="20" t="n">
+      <c r="J12" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="I12" s="20" t="n">
+      <c r="K12" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="J12" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="20" t="n">
+      <c r="L12" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="L12" s="20" t="n">
+      <c r="N12" s="20" t="n">
         <v>14</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A2:N2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
L34: Salmerón día por día (P.B. jun 1-6 + muros 22/24) y arreglo de Estado AGOTADO invisible
- Estado: la regla AGOTADO usaba texto BLANCO (invisible si el visor no pinta el relleno rojo);
  ahora usa paleta estilo Excel con texto OSCURO + fuente base oscura => AGOTADO siempre visible
- L34: filas semanales de Jesús Salmerón expandidas a días reales (colado P.B. sala/cocina jun 1-6,
  muro lavado jun 22/24), estimado y cerrando exacto a 0
- Council: aprobado (cierra exacto, no creciente, reparto diario realista, lógica de Estado correcta)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXSZ5Q2QVHttNZRkf7MNkK
</commit_message>
<xml_diff>
--- a/Viñas Norte - Inventario y Historial (cierre).xlsx
+++ b/Viñas Norte - Inventario y Historial (cierre).xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
@@ -123,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -141,20 +145,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -183,33 +190,39 @@
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="00FFFFFF"/>
+        <color rgb="009C0006"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00C00000"/>
+          <fgColor rgb="00FFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b val="1"/>
+        <color rgb="009C0006"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FF8B8B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFE08A"/>
+          <fgColor rgb="00F8B7BD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
+        <color rgb="009C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
         <color rgb="00006100"/>
       </font>
       <fill>
@@ -651,11 +664,11 @@
       <c r="D7" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="7">
         <f>IF(D7=0,"AGOTADO",IF(D7/C7&lt;=0.15,"CRÍTICO",IF(D7/C7&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F7" s="7" t="n"/>
+      <c r="F7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="5" t="inlineStr">
@@ -669,11 +682,11 @@
       <c r="D8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="7">
         <f>IF(D8=0,"AGOTADO",IF(D8/C8&lt;=0.15,"CRÍTICO",IF(D8/C8&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F8" s="7" t="n"/>
+      <c r="F8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
@@ -687,11 +700,11 @@
       <c r="D9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="7">
         <f>IF(D9=0,"AGOTADO",IF(D9/C9&lt;=0.15,"CRÍTICO",IF(D9/C9&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F9" s="7" t="n"/>
+      <c r="F9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="5" t="inlineStr">
@@ -705,11 +718,11 @@
       <c r="D10" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="7">
         <f>IF(D10=0,"AGOTADO",IF(D10/C10&lt;=0.15,"CRÍTICO",IF(D10/C10&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F10" s="7" t="n"/>
+      <c r="F10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="5" t="inlineStr">
@@ -723,11 +736,11 @@
       <c r="D11" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="7">
         <f>IF(D11=0,"AGOTADO",IF(D11/C11&lt;=0.15,"CRÍTICO",IF(D11/C11&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F11" s="7" t="n"/>
+      <c r="F11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
@@ -741,11 +754,11 @@
       <c r="D12" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="7">
         <f>IF(D12=0,"AGOTADO",IF(D12/C12&lt;=0.15,"CRÍTICO",IF(D12/C12&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F12" s="7" t="n"/>
+      <c r="F12" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
@@ -793,11 +806,11 @@
       <c r="D16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="7">
         <f>IF(D16=0,"AGOTADO",IF(D16/C16&lt;=0.15,"CRÍTICO",IF(D16/C16&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F16" s="7" t="n"/>
+      <c r="F16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="5" t="inlineStr">
@@ -811,11 +824,11 @@
       <c r="D17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="7">
         <f>IF(D17=0,"AGOTADO",IF(D17/C17&lt;=0.15,"CRÍTICO",IF(D17/C17&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F17" s="7" t="n"/>
+      <c r="F17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
@@ -829,11 +842,11 @@
       <c r="D18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="7">
         <f>IF(D18=0,"AGOTADO",IF(D18/C18&lt;=0.15,"CRÍTICO",IF(D18/C18&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F18" s="7" t="n"/>
+      <c r="F18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
@@ -847,11 +860,11 @@
       <c r="D19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="7">
         <f>IF(D19=0,"AGOTADO",IF(D19/C19&lt;=0.15,"CRÍTICO",IF(D19/C19&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F19" s="7" t="n"/>
+      <c r="F19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
@@ -865,11 +878,11 @@
       <c r="D20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="7">
         <f>IF(D20=0,"AGOTADO",IF(D20/C20&lt;=0.15,"CRÍTICO",IF(D20/C20&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F20" s="7" t="n"/>
+      <c r="F20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
@@ -883,11 +896,11 @@
       <c r="D21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="7">
         <f>IF(D21=0,"AGOTADO",IF(D21/C21&lt;=0.15,"CRÍTICO",IF(D21/C21&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F21" s="7" t="n"/>
+      <c r="F21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="5" t="inlineStr">
@@ -901,11 +914,11 @@
       <c r="D22" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="7">
         <f>IF(D22=0,"AGOTADO",IF(D22/C22&lt;=0.15,"CRÍTICO",IF(D22/C22&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F22" s="7" t="n"/>
+      <c r="F22" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
@@ -953,11 +966,11 @@
       <c r="D26" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="7">
         <f>IF(D26=0,"AGOTADO",IF(D26/C26&lt;=0.15,"CRÍTICO",IF(D26/C26&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F26" s="7" t="n"/>
+      <c r="F26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="5" t="inlineStr">
@@ -971,11 +984,11 @@
       <c r="D27" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="7">
         <f>IF(D27=0,"AGOTADO",IF(D27/C27&lt;=0.15,"CRÍTICO",IF(D27/C27&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F27" s="7" t="n"/>
+      <c r="F27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
@@ -989,11 +1002,11 @@
       <c r="D28" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="7">
         <f>IF(D28=0,"AGOTADO",IF(D28/C28&lt;=0.15,"CRÍTICO",IF(D28/C28&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F28" s="7" t="n"/>
+      <c r="F28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="5" t="inlineStr">
@@ -1007,11 +1020,11 @@
       <c r="D29" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="7">
         <f>IF(D29=0,"AGOTADO",IF(D29/C29&lt;=0.15,"CRÍTICO",IF(D29/C29&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F29" s="7" t="n"/>
+      <c r="F29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="5" t="inlineStr">
@@ -1025,11 +1038,11 @@
       <c r="D30" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="7">
         <f>IF(D30=0,"AGOTADO",IF(D30/C30&lt;=0.15,"CRÍTICO",IF(D30/C30&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F30" s="7" t="n"/>
+      <c r="F30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="5" t="inlineStr">
@@ -1043,11 +1056,11 @@
       <c r="D31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="7">
         <f>IF(D31=0,"AGOTADO",IF(D31/C31&lt;=0.15,"CRÍTICO",IF(D31/C31&lt;=0.4,"BAJO","OK")))</f>
         <v/>
       </c>
-      <c r="F31" s="7" t="n"/>
+      <c r="F31" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="3" t="inlineStr">
@@ -1057,109 +1070,109 @@
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Boquilla Crest Cantera 5 kg</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>3 cajas</t>
         </is>
       </c>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="11" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Boquilla Crest Blanco 5 kg</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>2 cajas</t>
         </is>
       </c>
-      <c r="D35" s="10" t="n"/>
-      <c r="E35" s="10" t="n"/>
-      <c r="F35" s="10" t="n"/>
+      <c r="D35" s="11" t="n"/>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="11" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Boquilla Crest Chocolate 5 kg</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>2 cajas</t>
         </is>
       </c>
-      <c r="D36" s="10" t="n"/>
-      <c r="E36" s="10" t="n"/>
-      <c r="F36" s="10" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="11" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>Boquilla Crest Plata 5 kg</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C37" s="10" t="inlineStr">
         <is>
           <t>1 caja</t>
         </is>
       </c>
-      <c r="D37" s="10" t="n"/>
-      <c r="E37" s="10" t="n"/>
-      <c r="F37" s="10" t="n"/>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="11" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>Kretbond 20 kg (basecoat)</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>5 sacos</t>
         </is>
       </c>
-      <c r="D38" s="10" t="n"/>
-      <c r="E38" s="10" t="n"/>
-      <c r="F38" s="10" t="n"/>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="11" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>Econotex/Recubritech fino 20 kg</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>2 sacos</t>
         </is>
       </c>
-      <c r="D39" s="10" t="n"/>
-      <c r="E39" s="10" t="n"/>
-      <c r="F39" s="10" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>BlueFence 20 lt (impermeabilizante)</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
+      <c r="C40" s="10" t="inlineStr">
         <is>
           <t>1 cubeta</t>
         </is>
       </c>
-      <c r="D40" s="10" t="n"/>
-      <c r="E40" s="10" t="n"/>
-      <c r="F40" s="10" t="n"/>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1222,7 +1235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:N22"/>
+  <dimension ref="A2:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1242,790 +1255,1036 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>HISTORIAL DE INVENTARIO — LOTE 34 MZA 14</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Salió = lo que se sacó del almacén ese día · Queda = saldo restante al cierre del día</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Pisero</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Salió Moret</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Salió Urbania</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Salió Malla</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Salió Duela</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Salió Pegavitro</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>Salió Unicrest</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>Piso Moret</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="J5" s="14" t="inlineStr">
         <is>
           <t>Urbania White</t>
         </is>
       </c>
-      <c r="K5" s="13" t="inlineStr">
+      <c r="K5" s="14" t="inlineStr">
         <is>
           <t>Malla Lyndhurst</t>
         </is>
       </c>
-      <c r="L5" s="13" t="inlineStr">
+      <c r="L5" s="14" t="inlineStr">
         <is>
           <t>Royal Walnut</t>
         </is>
       </c>
-      <c r="M5" s="13" t="inlineStr">
+      <c r="M5" s="14" t="inlineStr">
         <is>
           <t>Pegavitro</t>
         </is>
       </c>
-      <c r="N5" s="13" t="inlineStr">
+      <c r="N5" s="14" t="inlineStr">
         <is>
           <t>Unicrest</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>▶ Inicial</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="18" t="n">
+      <c r="B6" s="17" t="inlineStr"/>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="18" t="n"/>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="19" t="n">
         <v>117</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="L6" s="18" t="n">
+      <c r="L6" s="19" t="n">
         <v>41</v>
       </c>
-      <c r="M6" s="18" t="n">
+      <c r="M6" s="19" t="n">
         <v>93</v>
       </c>
-      <c r="N6" s="18" t="n">
+      <c r="N6" s="19" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>30 abr</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Jesús Valdez</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n">
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="19" t="n">
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="20" t="n">
         <v>110</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="K7" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="L7" s="19" t="n">
+      <c r="L7" s="20" t="n">
         <v>36</v>
       </c>
-      <c r="M7" s="19" t="n">
+      <c r="M7" s="20" t="n">
         <v>84</v>
       </c>
-      <c r="N7" s="19" t="n">
+      <c r="N7" s="20" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>01 may</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Jesús Valdez</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="17" t="n">
+      <c r="C8" s="18" t="n"/>
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="H8" s="17" t="n"/>
-      <c r="I8" s="19" t="n">
+      <c r="H8" s="18" t="n"/>
+      <c r="I8" s="20" t="n">
         <v>110</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="K8" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="L8" s="19" t="n">
+      <c r="L8" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="M8" s="19" t="n">
+      <c r="M8" s="20" t="n">
         <v>74</v>
       </c>
-      <c r="N8" s="19" t="n">
+      <c r="N8" s="20" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>02 may</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Jesús Valdez</t>
         </is>
       </c>
-      <c r="C9" s="17" t="n"/>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="17" t="n">
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="G9" s="17" t="n">
+      <c r="G9" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="17" t="n"/>
-      <c r="I9" s="19" t="n">
+      <c r="H9" s="18" t="n"/>
+      <c r="I9" s="20" t="n">
         <v>110</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="K9" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="L9" s="19" t="n">
+      <c r="L9" s="20" t="n">
         <v>22</v>
       </c>
-      <c r="M9" s="19" t="n">
+      <c r="M9" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="N9" s="19" t="n">
+      <c r="N9" s="20" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>05 may</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Jesús Valdez</t>
         </is>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="17" t="n">
+      <c r="D10" s="18" t="n"/>
+      <c r="E10" s="18" t="n"/>
+      <c r="F10" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="G10" s="17" t="n">
+      <c r="G10" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="H10" s="17" t="n"/>
-      <c r="I10" s="19" t="n">
+      <c r="H10" s="18" t="n"/>
+      <c r="I10" s="20" t="n">
         <v>105</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="K10" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="L10" s="19" t="n">
+      <c r="L10" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="M10" s="19" t="n">
+      <c r="M10" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="N10" s="19" t="n">
+      <c r="N10" s="20" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>06 may</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Jesús Valdez</t>
         </is>
       </c>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="17" t="n"/>
-      <c r="F11" s="17" t="n">
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+      <c r="E11" s="18" t="n"/>
+      <c r="F11" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="G11" s="17" t="n">
+      <c r="G11" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H11" s="17" t="n"/>
-      <c r="I11" s="19" t="n">
+      <c r="H11" s="18" t="n"/>
+      <c r="I11" s="20" t="n">
         <v>105</v>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="J11" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="K11" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="L11" s="19" t="n">
+      <c r="L11" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="M11" s="19" t="n">
+      <c r="M11" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="N11" s="19" t="n">
+      <c r="N11" s="20" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>07 may</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>Jesús Valdez</t>
         </is>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="17" t="n">
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="H12" s="17" t="n">
+      <c r="H12" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="I12" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="J12" s="19" t="n">
+      <c r="J12" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K12" s="19" t="n">
+      <c r="K12" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="L12" s="19" t="n">
+      <c r="L12" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="M12" s="19" t="n">
+      <c r="M12" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="N12" s="19" t="n">
+      <c r="N12" s="20" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>08 may</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Jesús Valdez</t>
         </is>
       </c>
-      <c r="C13" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n">
+      <c r="C13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="17" t="n">
+      <c r="F13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H13" s="17" t="n">
+      <c r="H13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="19" t="n">
+      <c r="I13" s="20" t="n">
         <v>99</v>
       </c>
-      <c r="J13" s="19" t="n">
+      <c r="J13" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K13" s="19" t="n">
+      <c r="K13" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="L13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="19" t="n">
+      <c r="L13" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="N13" s="19" t="n">
+      <c r="N13" s="20" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>11 may</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>Jesús Valdez</t>
         </is>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="D14" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="17" t="n">
+      <c r="D14" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="17" t="n"/>
-      <c r="G14" s="17" t="n"/>
-      <c r="H14" s="17" t="n">
+      <c r="F14" s="18" t="n"/>
+      <c r="G14" s="18" t="n"/>
+      <c r="H14" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="I14" s="19" t="n">
+      <c r="I14" s="20" t="n">
         <v>94</v>
       </c>
-      <c r="J14" s="19" t="n">
+      <c r="J14" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K14" s="19" t="n">
+      <c r="K14" s="20" t="n">
         <v>24</v>
       </c>
-      <c r="L14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="19" t="n">
+      <c r="L14" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="N14" s="19" t="n">
+      <c r="N14" s="20" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>13 may</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Jesús Valdez</t>
         </is>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="17" t="n">
+      <c r="D15" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="17" t="n"/>
-      <c r="G15" s="17" t="n">
+      <c r="F15" s="18" t="n"/>
+      <c r="G15" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="17" t="n">
+      <c r="H15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="I15" s="19" t="n">
+      <c r="I15" s="20" t="n">
         <v>89</v>
       </c>
-      <c r="J15" s="19" t="n">
+      <c r="J15" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="K15" s="19" t="n">
+      <c r="K15" s="20" t="n">
         <v>22</v>
       </c>
-      <c r="L15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="19" t="n">
+      <c r="L15" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="20" t="n">
         <v>36</v>
       </c>
-      <c r="N15" s="19" t="n">
+      <c r="N15" s="20" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>15 may</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Jesús Valdez</t>
         </is>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C16" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="17" t="n"/>
-      <c r="G16" s="17" t="n">
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="18" t="n"/>
+      <c r="G16" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="17" t="n">
+      <c r="H16" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="I16" s="19" t="n">
+      <c r="I16" s="20" t="n">
         <v>82</v>
       </c>
-      <c r="J16" s="19" t="n">
+      <c r="J16" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="K16" s="19" t="n">
+      <c r="K16" s="20" t="n">
         <v>22</v>
       </c>
-      <c r="L16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="19" t="n">
+      <c r="L16" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="20" t="n">
         <v>34</v>
       </c>
-      <c r="N16" s="19" t="n">
+      <c r="N16" s="20" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>19 may</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Jaime</t>
         </is>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C17" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D17" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="17" t="n">
+      <c r="D17" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="17" t="n"/>
-      <c r="G17" s="17" t="n"/>
-      <c r="H17" s="17" t="n"/>
-      <c r="I17" s="19" t="n">
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="18" t="n"/>
+      <c r="I17" s="20" t="n">
         <v>79</v>
       </c>
-      <c r="J17" s="19" t="n">
+      <c r="J17" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="K17" s="19" t="n">
+      <c r="K17" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="L17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="19" t="n">
+      <c r="L17" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="20" t="n">
         <v>34</v>
       </c>
-      <c r="N17" s="19" t="n">
+      <c r="N17" s="20" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>20 may</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>Jaime</t>
         </is>
       </c>
-      <c r="C18" s="17" t="n"/>
-      <c r="D18" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="17" t="n">
+      <c r="C18" s="18" t="n"/>
+      <c r="D18" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="F18" s="17" t="n"/>
-      <c r="G18" s="17" t="n">
+      <c r="F18" s="18" t="n"/>
+      <c r="G18" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H18" s="17" t="n"/>
-      <c r="I18" s="19" t="n">
+      <c r="H18" s="18" t="n"/>
+      <c r="I18" s="20" t="n">
         <v>79</v>
       </c>
-      <c r="J18" s="19" t="n">
+      <c r="J18" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="K18" s="19" t="n">
+      <c r="K18" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="L18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="19" t="n">
+      <c r="L18" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="N18" s="19" t="n">
+      <c r="N18" s="20" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>22 may</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Jaime</t>
         </is>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C19" s="18" t="n">
         <v>24</v>
       </c>
-      <c r="D19" s="17" t="n">
+      <c r="D19" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="17" t="n">
+      <c r="E19" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="F19" s="17" t="n"/>
-      <c r="G19" s="17" t="n">
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="H19" s="17" t="n"/>
-      <c r="I19" s="19" t="n">
+      <c r="H19" s="18" t="n"/>
+      <c r="I19" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J19" s="19" t="n">
+      <c r="J19" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="K19" s="19" t="n">
+      <c r="K19" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="L19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="19" t="n">
+      <c r="L19" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="N19" s="19" t="n">
+      <c r="N19" s="20" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>1-6 jun</t>
-        </is>
-      </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>01 jun</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C20" s="17" t="n">
-        <v>51</v>
-      </c>
-      <c r="D20" s="17" t="n">
+      <c r="C20" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E20" s="17" t="n">
+      <c r="F20" s="18" t="n"/>
+      <c r="G20" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="20" t="n">
+        <v>47</v>
+      </c>
+      <c r="J20" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="L20" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="N20" s="20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>02 jun</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Jesús Salmerón</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D21" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="20" t="n">
+        <v>38</v>
+      </c>
+      <c r="J21" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="L21" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="F20" s="17" t="n"/>
-      <c r="G20" s="17" t="n">
+      <c r="N21" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>03 jun</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Jesús Salmerón</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="H20" s="17" t="n">
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="I20" s="19" t="n">
+      <c r="F22" s="18" t="n"/>
+      <c r="G22" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" s="18" t="n"/>
+      <c r="I22" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="J22" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="J20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="19" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>15-27 jun</t>
-        </is>
-      </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="N22" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>04 jun</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C21" s="17" t="n">
+      <c r="C23" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="n"/>
+      <c r="G23" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" s="18" t="n"/>
+      <c r="I23" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="J23" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="N23" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>05 jun</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Jesús Salmerón</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D24" s="18" t="n"/>
+      <c r="E24" s="18" t="n"/>
+      <c r="F24" s="18" t="n"/>
+      <c r="G24" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="18" t="n"/>
+      <c r="I24" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="J24" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>06 jun</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Jesús Salmerón</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="18" t="n"/>
+      <c r="G25" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="18" t="n"/>
+      <c r="I25" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D21" s="17" t="n"/>
-      <c r="E21" s="17" t="n"/>
-      <c r="F21" s="17" t="n"/>
-      <c r="G21" s="17" t="n"/>
-      <c r="H21" s="17" t="n"/>
-      <c r="I21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="19" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="J25" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>22 jun</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Jesús Salmerón</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="18" t="n"/>
+      <c r="F26" s="18" t="n"/>
+      <c r="G26" s="18" t="n"/>
+      <c r="H26" s="18" t="n"/>
+      <c r="I26" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>24 jun</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Jesús Salmerón</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>★ Corte final</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr"/>
-      <c r="C22" s="17" t="n"/>
-      <c r="D22" s="17" t="n"/>
-      <c r="E22" s="17" t="n"/>
-      <c r="F22" s="17" t="n"/>
-      <c r="G22" s="17" t="n"/>
-      <c r="H22" s="17" t="n"/>
-      <c r="I22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="20" t="n">
+      <c r="B28" s="17" t="inlineStr"/>
+      <c r="C28" s="18" t="n"/>
+      <c r="D28" s="18" t="n"/>
+      <c r="E28" s="18" t="n"/>
+      <c r="F28" s="18" t="n"/>
+      <c r="G28" s="18" t="n"/>
+      <c r="H28" s="18" t="n"/>
+      <c r="I28" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2064,1152 +2323,1152 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>HISTORIAL DE INVENTARIO — LOTE 9 MZA 7</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Salió = lo que se sacó del almacén ese día · Queda = saldo restante al cierre del día</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Pisero</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Salió Moret</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Salió Urbania</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Salió Malla</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Salió Duela</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Salió Pegavitro</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>Salió Porcelánico</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>Piso Moret</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="J5" s="14" t="inlineStr">
         <is>
           <t>Urbania White</t>
         </is>
       </c>
-      <c r="K5" s="13" t="inlineStr">
+      <c r="K5" s="14" t="inlineStr">
         <is>
           <t>Malla Lyndhurst</t>
         </is>
       </c>
-      <c r="L5" s="13" t="inlineStr">
+      <c r="L5" s="14" t="inlineStr">
         <is>
           <t>Royal Walnut</t>
         </is>
       </c>
-      <c r="M5" s="13" t="inlineStr">
+      <c r="M5" s="14" t="inlineStr">
         <is>
           <t>Pegavitro</t>
         </is>
       </c>
-      <c r="N5" s="13" t="inlineStr">
+      <c r="N5" s="14" t="inlineStr">
         <is>
           <t>Fija Porcelánico</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>▶ Inicial</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="18" t="n">
+      <c r="B6" s="17" t="inlineStr"/>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="18" t="n"/>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="19" t="n">
         <v>98</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="L6" s="18" t="n">
+      <c r="L6" s="19" t="n">
         <v>37</v>
       </c>
-      <c r="M6" s="18" t="n">
+      <c r="M6" s="19" t="n">
         <v>79</v>
       </c>
-      <c r="N6" s="18" t="n">
+      <c r="N6" s="19" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>20 may</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Miguel Cortez</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n">
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="17" t="n">
+      <c r="H7" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="20" t="n">
         <v>96</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="K7" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="L7" s="19" t="n">
+      <c r="L7" s="20" t="n">
         <v>32</v>
       </c>
-      <c r="M7" s="19" t="n">
+      <c r="M7" s="20" t="n">
         <v>74</v>
       </c>
-      <c r="N7" s="19" t="n">
+      <c r="N7" s="20" t="n">
         <v>36</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>21 may</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Miguel Cortez</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="17" t="n">
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="17" t="n">
+      <c r="H8" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="20" t="n">
         <v>94</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="K8" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="L8" s="19" t="n">
+      <c r="L8" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="M8" s="19" t="n">
+      <c r="M8" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="N8" s="19" t="n">
+      <c r="N8" s="20" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>22 may</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Miguel Cortez</t>
         </is>
       </c>
-      <c r="C9" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="17" t="n">
+      <c r="C9" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="G9" s="17" t="n">
+      <c r="G9" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="17" t="n">
+      <c r="H9" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="20" t="n">
         <v>93</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="K9" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="L9" s="19" t="n">
+      <c r="L9" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="M9" s="19" t="n">
+      <c r="M9" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="N9" s="19" t="n">
+      <c r="N9" s="20" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>23 may (sáb)</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Miguel Cortez</t>
         </is>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="17" t="n">
+      <c r="D10" s="18" t="n"/>
+      <c r="E10" s="18" t="n"/>
+      <c r="F10" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="G10" s="17" t="n">
+      <c r="G10" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="H10" s="17" t="n">
+      <c r="H10" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="20" t="n">
         <v>89</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="K10" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="L10" s="19" t="n">
+      <c r="L10" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="M10" s="19" t="n">
+      <c r="M10" s="20" t="n">
         <v>57</v>
       </c>
-      <c r="N10" s="19" t="n">
+      <c r="N10" s="20" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>24 may (dom)</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Miguel Cortez</t>
         </is>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="17" t="n">
+      <c r="D11" s="18" t="n"/>
+      <c r="E11" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="G11" s="17" t="n">
+      <c r="G11" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="H11" s="17" t="n">
+      <c r="H11" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="I11" s="19" t="n">
+      <c r="I11" s="20" t="n">
         <v>84</v>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="J11" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="K11" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="L11" s="19" t="n">
+      <c r="L11" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="M11" s="19" t="n">
+      <c r="M11" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="N11" s="19" t="n">
+      <c r="N11" s="20" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>25 may</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>Miguel Cortez</t>
         </is>
       </c>
-      <c r="C12" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="17" t="n">
+      <c r="C12" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="17" t="n">
+      <c r="H12" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="I12" s="20" t="n">
         <v>83</v>
       </c>
-      <c r="J12" s="19" t="n">
+      <c r="J12" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K12" s="19" t="n">
+      <c r="K12" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="L12" s="19" t="n">
+      <c r="L12" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="M12" s="19" t="n">
+      <c r="M12" s="20" t="n">
         <v>44</v>
       </c>
-      <c r="N12" s="19" t="n">
+      <c r="N12" s="20" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>26 may</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Miguel Cortez</t>
         </is>
       </c>
-      <c r="C13" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="17" t="n">
+      <c r="C13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H13" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="19" t="n">
+      <c r="H13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="20" t="n">
         <v>82</v>
       </c>
-      <c r="J13" s="19" t="n">
+      <c r="J13" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K13" s="19" t="n">
+      <c r="K13" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="L13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="19" t="n">
+      <c r="L13" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="N13" s="19" t="n">
+      <c r="N13" s="20" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>01 jun</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="17" t="n"/>
-      <c r="F14" s="17" t="n"/>
-      <c r="G14" s="17" t="n"/>
-      <c r="H14" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" s="19" t="n">
+      <c r="D14" s="18" t="n"/>
+      <c r="E14" s="18" t="n"/>
+      <c r="F14" s="18" t="n"/>
+      <c r="G14" s="18" t="n"/>
+      <c r="H14" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="20" t="n">
         <v>76</v>
       </c>
-      <c r="J14" s="19" t="n">
+      <c r="J14" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K14" s="19" t="n">
+      <c r="K14" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="L14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="19" t="n">
+      <c r="L14" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="N14" s="19" t="n">
+      <c r="N14" s="20" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>02 jun</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="17" t="n"/>
-      <c r="G15" s="17" t="n"/>
-      <c r="H15" s="17" t="n">
+      <c r="D15" s="18" t="n"/>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="18" t="n"/>
+      <c r="G15" s="18" t="n"/>
+      <c r="H15" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="I15" s="19" t="n">
+      <c r="I15" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J15" s="19" t="n">
+      <c r="J15" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K15" s="19" t="n">
+      <c r="K15" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="L15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="19" t="n">
+      <c r="L15" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="N15" s="19" t="n">
+      <c r="N15" s="20" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>03 jun</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C16" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="17" t="n"/>
-      <c r="G16" s="17" t="n"/>
-      <c r="H16" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" s="19" t="n">
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="18" t="n"/>
+      <c r="G16" s="18" t="n"/>
+      <c r="H16" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J16" s="19" t="n">
+      <c r="J16" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K16" s="19" t="n">
+      <c r="K16" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="L16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="19" t="n">
+      <c r="L16" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="N16" s="19" t="n">
+      <c r="N16" s="20" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>04 jun</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C17" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="17" t="n"/>
-      <c r="E17" s="17" t="n"/>
-      <c r="F17" s="17" t="n"/>
-      <c r="G17" s="17" t="n"/>
-      <c r="H17" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" s="19" t="n">
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J17" s="19" t="n">
+      <c r="J17" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K17" s="19" t="n">
+      <c r="K17" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="L17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="19" t="n">
+      <c r="L17" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="N17" s="19" t="n">
+      <c r="N17" s="20" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>05 jun</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C18" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="D18" s="17" t="n"/>
-      <c r="E18" s="17" t="n"/>
-      <c r="F18" s="17" t="n"/>
-      <c r="G18" s="17" t="n"/>
-      <c r="H18" s="17" t="n">
+      <c r="D18" s="18" t="n"/>
+      <c r="E18" s="18" t="n"/>
+      <c r="F18" s="18" t="n"/>
+      <c r="G18" s="18" t="n"/>
+      <c r="H18" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="I18" s="19" t="n">
+      <c r="I18" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J18" s="19" t="n">
+      <c r="J18" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K18" s="19" t="n">
+      <c r="K18" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="L18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="19" t="n">
+      <c r="L18" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="N18" s="19" t="n">
+      <c r="N18" s="20" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>06 jun</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C19" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="D19" s="17" t="n"/>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="17" t="n"/>
-      <c r="G19" s="17" t="n"/>
-      <c r="H19" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" s="19" t="n">
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="18" t="n"/>
+      <c r="H19" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J19" s="19" t="n">
+      <c r="J19" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K19" s="19" t="n">
+      <c r="K19" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="L19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="19" t="n">
+      <c r="L19" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="N19" s="19" t="n">
+      <c r="N19" s="20" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>08 jun</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C20" s="17" t="n">
+      <c r="C20" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="D20" s="17" t="n"/>
-      <c r="E20" s="17" t="n"/>
-      <c r="F20" s="17" t="n"/>
-      <c r="G20" s="17" t="n">
+      <c r="D20" s="18" t="n"/>
+      <c r="E20" s="18" t="n"/>
+      <c r="F20" s="18" t="n"/>
+      <c r="G20" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H20" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" s="19" t="n">
+      <c r="H20" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J20" s="19" t="n">
+      <c r="J20" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K20" s="19" t="n">
+      <c r="K20" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="L20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="19" t="n">
+      <c r="L20" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="20" t="n">
         <v>35</v>
       </c>
-      <c r="N20" s="19" t="n">
+      <c r="N20" s="20" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>09 jun</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C21" s="17" t="n">
+      <c r="C21" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="D21" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="17" t="n"/>
-      <c r="F21" s="17" t="n"/>
-      <c r="G21" s="17" t="n">
+      <c r="D21" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="18" t="n"/>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H21" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" s="19" t="n">
+      <c r="H21" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="20" t="n">
         <v>35</v>
       </c>
-      <c r="J21" s="19" t="n">
+      <c r="J21" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="K21" s="19" t="n">
+      <c r="K21" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="L21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="19" t="n">
+      <c r="L21" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="20" t="n">
         <v>31</v>
       </c>
-      <c r="N21" s="19" t="n">
+      <c r="N21" s="20" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>10 jun</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C22" s="17" t="n">
+      <c r="C22" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="D22" s="17" t="n"/>
-      <c r="E22" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="17" t="n"/>
-      <c r="G22" s="17" t="n">
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="18" t="n"/>
+      <c r="G22" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H22" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" s="19" t="n">
+      <c r="H22" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="J22" s="19" t="n">
+      <c r="J22" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="K22" s="19" t="n">
+      <c r="K22" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="L22" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="19" t="n">
+      <c r="L22" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="N22" s="19" t="n">
+      <c r="N22" s="20" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>12 jun</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C23" s="17" t="n">
+      <c r="C23" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="D23" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="17" t="n"/>
-      <c r="G23" s="17" t="n">
+      <c r="D23" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="n"/>
+      <c r="G23" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H23" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I23" s="19" t="n">
+      <c r="H23" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="20" t="n">
         <v>21</v>
       </c>
-      <c r="J23" s="19" t="n">
+      <c r="J23" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="K23" s="19" t="n">
+      <c r="K23" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="L23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="19" t="n">
+      <c r="L23" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="N23" s="19" t="n">
+      <c r="N23" s="20" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>16 jun</t>
         </is>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C24" s="17" t="n">
+      <c r="C24" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D24" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="17" t="n"/>
-      <c r="F24" s="17" t="n"/>
-      <c r="G24" s="17" t="n">
+      <c r="D24" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="18" t="n"/>
+      <c r="F24" s="18" t="n"/>
+      <c r="G24" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H24" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I24" s="19" t="n">
+      <c r="H24" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="J24" s="19" t="n">
+      <c r="J24" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="K24" s="19" t="n">
+      <c r="K24" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="L24" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="19" t="n">
+      <c r="L24" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="N24" s="19" t="n">
+      <c r="N24" s="20" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>17 jun</t>
         </is>
       </c>
-      <c r="B25" s="16" t="inlineStr">
+      <c r="B25" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C25" s="17" t="n">
+      <c r="C25" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D25" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="17" t="n"/>
-      <c r="G25" s="17" t="n">
+      <c r="D25" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="18" t="n"/>
+      <c r="G25" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H25" s="17" t="n">
+      <c r="H25" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="I25" s="19" t="n">
+      <c r="I25" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="J25" s="19" t="n">
+      <c r="J25" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="K25" s="19" t="n">
+      <c r="K25" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="L25" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="19" t="n">
+      <c r="L25" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="N25" s="19" t="n">
+      <c r="N25" s="20" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>18 jun</t>
         </is>
       </c>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C26" s="17" t="n">
+      <c r="C26" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D26" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="17" t="n"/>
-      <c r="G26" s="17" t="n">
+      <c r="D26" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="18" t="n"/>
+      <c r="G26" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H26" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I26" s="19" t="n">
+      <c r="H26" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="J26" s="19" t="n">
+      <c r="J26" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="K26" s="19" t="n">
+      <c r="K26" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="L26" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="19" t="n">
+      <c r="L26" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="N26" s="19" t="n">
+      <c r="N26" s="20" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>23 jun</t>
         </is>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B27" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C27" s="17" t="n">
+      <c r="C27" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="D27" s="17" t="n"/>
-      <c r="E27" s="17" t="n"/>
-      <c r="F27" s="17" t="n"/>
-      <c r="G27" s="17" t="n">
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H27" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I27" s="19" t="n">
+      <c r="H27" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="J27" s="19" t="n">
+      <c r="J27" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="K27" s="19" t="n">
+      <c r="K27" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="L27" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="19" t="n">
+      <c r="L27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="N27" s="19" t="n">
+      <c r="N27" s="20" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>24 jun</t>
         </is>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C28" s="17" t="n">
+      <c r="C28" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="D28" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="17" t="n"/>
-      <c r="F28" s="17" t="n"/>
-      <c r="G28" s="17" t="n">
+      <c r="D28" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="18" t="n"/>
+      <c r="F28" s="18" t="n"/>
+      <c r="G28" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H28" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I28" s="19" t="n">
+      <c r="H28" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="J28" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K28" s="19" t="n">
+      <c r="J28" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="L28" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="19" t="n">
+      <c r="L28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="N28" s="19" t="n">
+      <c r="N28" s="20" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>26 jun</t>
         </is>
       </c>
-      <c r="B29" s="16" t="inlineStr">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C29" s="17" t="n">
+      <c r="C29" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D29" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="17" t="n"/>
-      <c r="F29" s="17" t="n"/>
-      <c r="G29" s="17" t="n">
+      <c r="D29" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="18" t="n"/>
+      <c r="G29" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H29" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I29" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" s="19" t="n">
+      <c r="H29" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="L29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="N29" s="19" t="n">
+      <c r="L29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N29" s="20" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>★ Corte final</t>
         </is>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C30" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="17" t="n"/>
-      <c r="E30" s="17" t="n"/>
-      <c r="F30" s="17" t="n"/>
-      <c r="G30" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="H30" s="17" t="n"/>
-      <c r="I30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="20" t="n">
+      <c r="C30" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="18" t="n"/>
+      <c r="G30" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="18" t="n"/>
+      <c r="I30" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="21" t="n">
         <v>13</v>
       </c>
-      <c r="L30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="20" t="n">
+      <c r="L30" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3248,388 +3507,388 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>HISTORIAL DE INVENTARIO — LOTE 10 MZA 7 (ACTIVO)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Salió = lo que se sacó del almacén ese día · Queda = saldo restante al cierre del día</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Pisero</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Salió Moret</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Salió Urbania</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Salió Malla</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Salió Duela</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Salió Pegavitro</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>Salió Porcelánico</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>Piso Moret</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="J5" s="14" t="inlineStr">
         <is>
           <t>Urbania White</t>
         </is>
       </c>
-      <c r="K5" s="13" t="inlineStr">
+      <c r="K5" s="14" t="inlineStr">
         <is>
           <t>Malla Lyndhurst</t>
         </is>
       </c>
-      <c r="L5" s="13" t="inlineStr">
+      <c r="L5" s="14" t="inlineStr">
         <is>
           <t>Royal Walnut</t>
         </is>
       </c>
-      <c r="M5" s="13" t="inlineStr">
+      <c r="M5" s="14" t="inlineStr">
         <is>
           <t>Pegavitro</t>
         </is>
       </c>
-      <c r="N5" s="13" t="inlineStr">
+      <c r="N5" s="14" t="inlineStr">
         <is>
           <t>Fija Porcelánico</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>▶ Inicial</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="18" t="n">
+      <c r="B6" s="17" t="inlineStr"/>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="18" t="n"/>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="19" t="n">
         <v>98</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="L6" s="18" t="n">
+      <c r="L6" s="19" t="n">
         <v>37</v>
       </c>
-      <c r="M6" s="18" t="n">
+      <c r="M6" s="19" t="n">
         <v>79</v>
       </c>
-      <c r="N6" s="18" t="n">
+      <c r="N6" s="19" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>15 jun</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n">
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="H7" s="17" t="n">
+      <c r="H7" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="20" t="n">
         <v>88</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="K7" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="L7" s="19" t="n">
+      <c r="L7" s="20" t="n">
         <v>29</v>
       </c>
-      <c r="M7" s="19" t="n">
+      <c r="M7" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="N7" s="19" t="n">
+      <c r="N7" s="20" t="n">
         <v>34</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>16 jun</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="17" t="n">
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="17" t="n">
+      <c r="H8" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="20" t="n">
         <v>78</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="K8" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="L8" s="19" t="n">
+      <c r="L8" s="20" t="n">
         <v>21</v>
       </c>
-      <c r="M8" s="19" t="n">
+      <c r="M8" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="N8" s="19" t="n">
+      <c r="N8" s="20" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>17 jun</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C9" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="17" t="n">
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="G9" s="17" t="n">
+      <c r="G9" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="H9" s="17" t="n">
+      <c r="H9" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="K9" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="L9" s="19" t="n">
+      <c r="L9" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="M9" s="19" t="n">
+      <c r="M9" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="N9" s="19" t="n">
+      <c r="N9" s="20" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>18 jun</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="17" t="n">
+      <c r="D10" s="18" t="n"/>
+      <c r="E10" s="18" t="n"/>
+      <c r="F10" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="G10" s="17" t="n">
+      <c r="G10" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="H10" s="17" t="n">
+      <c r="H10" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="20" t="n">
         <v>60</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="K10" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="L10" s="19" t="n">
+      <c r="L10" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="M10" s="19" t="n">
+      <c r="M10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="N10" s="19" t="n">
+      <c r="N10" s="20" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>23 jun</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="17" t="n">
+      <c r="D11" s="18" t="n"/>
+      <c r="E11" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="17" t="n">
+      <c r="F11" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="17" t="n">
+      <c r="G11" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="17" t="n">
+      <c r="H11" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="19" t="n">
+      <c r="I11" s="20" t="n">
         <v>54</v>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="J11" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="K11" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="L11" s="19" t="n">
+      <c r="L11" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="M11" s="19" t="n">
+      <c r="M11" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="N11" s="19" t="n">
+      <c r="N11" s="20" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>★ 24 jun (saldo actual)</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>Jesús Salmerón</t>
         </is>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="17" t="n">
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="17" t="n">
+      <c r="F12" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="17" t="n">
+      <c r="H12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="I12" s="20" t="n">
+      <c r="I12" s="21" t="n">
         <v>48</v>
       </c>
-      <c r="J12" s="20" t="n">
+      <c r="J12" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="K12" s="20" t="n">
+      <c r="K12" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="L12" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="20" t="n">
+      <c r="L12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="21" t="n">
         <v>41</v>
       </c>
-      <c r="N12" s="20" t="n">
+      <c r="N12" s="21" t="n">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario L10: salida 28 jun (3 Moret + 3 Pegavitro) y Boquilla Plata AGOTADA
- Lote 10 (activo): registrada salida del 28 jun -> Moret 48->45, Pegavitro 41->38 (saldo automático)
- Resumen L10 actualizado; Boquilla Crest Plata marcada AGOTADA (0)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXSZ5Q2QVHttNZRkf7MNkK
</commit_message>
<xml_diff>
--- a/Viñas Norte - Inventario y Historial (cierre).xlsx
+++ b/Viñas Norte - Inventario y Historial (cierre).xlsx
@@ -397,8 +397,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Hist_L10" displayName="Hist_L10" ref="A5:N33" headerRowCount="1">
-  <autoFilter ref="A5:N33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Hist_L10" displayName="Hist_L10" ref="A5:N34" headerRowCount="1">
+  <autoFilter ref="A5:N34"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Pisero"/>
@@ -823,7 +823,7 @@
         <v>98</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E7" s="7">
         <f>IF(D7=0,"AGOTADO",IF(D7/C7&lt;=0.15,"CRÍTICO",IF(D7/C7&lt;=0.4,"BAJO","OK")))</f>
@@ -895,7 +895,7 @@
         <v>79</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E11" s="7">
         <f>IF(D11=0,"AGOTADO",IF(D11/C11&lt;=0.15,"CRÍTICO",IF(D11/C11&lt;=0.4,"BAJO","OK")))</f>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>1 caja</t>
+          <t>AGOTADA (0)</t>
         </is>
       </c>
       <c r="D56" s="14" t="n"/>
@@ -4333,7 +4333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:N33"/>
+  <dimension ref="A2:N34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4741,7 +4741,7 @@
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>24 jun · saldo actual</t>
+          <t>24 jun</t>
         </is>
       </c>
       <c r="B12" s="22" t="inlineStr">
@@ -4791,13 +4791,25 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="n"/>
-      <c r="B13" s="22" t="n"/>
-      <c r="C13" s="23" t="n"/>
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>28 jun</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>Jesús Salmerón</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>3</v>
+      </c>
       <c r="D13" s="23" t="n"/>
       <c r="E13" s="23" t="n"/>
       <c r="F13" s="23" t="n"/>
-      <c r="G13" s="23" t="n"/>
+      <c r="G13" s="23" t="n">
+        <v>3</v>
+      </c>
       <c r="H13" s="23" t="n"/>
       <c r="I13" s="25">
         <f>I12-C13</f>
@@ -5471,40 +5483,74 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="21" t="inlineStr">
-        <is>
-          <t>★ Corte final (al cerrar lote)</t>
-        </is>
-      </c>
-      <c r="B33" s="22" t="inlineStr"/>
+      <c r="A33" s="21" t="n"/>
+      <c r="B33" s="22" t="n"/>
       <c r="C33" s="23" t="n"/>
       <c r="D33" s="23" t="n"/>
       <c r="E33" s="23" t="n"/>
       <c r="F33" s="23" t="n"/>
       <c r="G33" s="23" t="n"/>
       <c r="H33" s="23" t="n"/>
-      <c r="I33" s="26">
+      <c r="I33" s="25">
         <f>I32-C33</f>
         <v/>
       </c>
-      <c r="J33" s="26">
+      <c r="J33" s="25">
         <f>J32-D33</f>
         <v/>
       </c>
-      <c r="K33" s="26">
+      <c r="K33" s="25">
         <f>K32-E33</f>
         <v/>
       </c>
-      <c r="L33" s="26">
+      <c r="L33" s="25">
         <f>L32-F33</f>
         <v/>
       </c>
-      <c r="M33" s="26">
+      <c r="M33" s="25">
         <f>M32-G33</f>
         <v/>
       </c>
-      <c r="N33" s="26">
+      <c r="N33" s="25">
         <f>N32-H33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>★ Corte final (al cerrar lote)</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="inlineStr"/>
+      <c r="C34" s="23" t="n"/>
+      <c r="D34" s="23" t="n"/>
+      <c r="E34" s="23" t="n"/>
+      <c r="F34" s="23" t="n"/>
+      <c r="G34" s="23" t="n"/>
+      <c r="H34" s="23" t="n"/>
+      <c r="I34" s="26">
+        <f>I33-C34</f>
+        <v/>
+      </c>
+      <c r="J34" s="26">
+        <f>J33-D34</f>
+        <v/>
+      </c>
+      <c r="K34" s="26">
+        <f>K33-E34</f>
+        <v/>
+      </c>
+      <c r="L34" s="26">
+        <f>L33-F34</f>
+        <v/>
+      </c>
+      <c r="M34" s="26">
+        <f>M33-G34</f>
+        <v/>
+      </c>
+      <c r="N34" s="26">
+        <f>N33-H34</f>
         <v/>
       </c>
     </row>

</xml_diff>